<commit_message>
Update automat catalog: 27.09.2026 21:32
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centralizator Medii" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cultură Generală" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module Tehnologice" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absențe &amp; Purtare" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fișă Individuală Elev" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adeverință Elev" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raport Diriginte" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Centralizator Medii" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cultură Generală" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Module Tehnologice" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Absențe &amp; Purtare" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fișă Individuală Elev" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Adeverință Elev" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Raport Diriginte" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -691,13 +691,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -721,7 +721,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -749,8 +749,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -776,8 +776,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -803,7 +803,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -818,9 +818,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -7934,10 +7934,22 @@
         <f>IF(SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9)=0, "", SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9))</f>
         <v/>
       </c>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="79" t="n"/>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="79" t="n"/>
+      <c r="H9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="79" t="inlineStr">
+        <is>
+          <t>27.09</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" s="79" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="n"/>
       <c r="M9" s="79" t="n"/>
       <c r="N9" s="6" t="n"/>
@@ -7996,8 +8008,14 @@
         <f>IF(COUNTA(AC9:BF9)=0, "", COUNTA(AC9:BF9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", AC9:BF9))))</f>
         <v/>
       </c>
-      <c r="BI9" s="79" t="n"/>
-      <c r="BJ9" s="79" t="n"/>
+      <c r="BI9" s="79" t="n">
+        <v>10</v>
+      </c>
+      <c r="BJ9" s="79" t="inlineStr">
+        <is>
+          <t>27.09</t>
+        </is>
+      </c>
       <c r="BK9" s="79" t="n"/>
       <c r="BL9" s="79" t="n"/>
       <c r="BM9" s="79" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 27.09.2026 21:51
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -7970,7 +7970,11 @@
         <f>IFERROR(ROUND(AVERAGE(H9,J9,L9,N9,P9,R9,T9,V9,X9,Z9), 2), "")</f>
         <v/>
       </c>
-      <c r="AC9" s="6" t="n"/>
+      <c r="AC9" s="79" t="inlineStr">
+        <is>
+          <t>27.09</t>
+        </is>
+      </c>
       <c r="AD9" s="79" t="n"/>
       <c r="AE9" s="6" t="n"/>
       <c r="AF9" s="79" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 27.09.2026 22:07
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -8688,8 +8688,14 @@
         <f>IF(COUNTA(WN9:XQ9)=0, "", COUNTA(WN9:XQ9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", WN9:XQ9))))</f>
         <v/>
       </c>
-      <c r="XT9" s="6" t="n"/>
-      <c r="XU9" s="6" t="n"/>
+      <c r="XT9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="XU9" s="79" t="inlineStr">
+        <is>
+          <t>27.09</t>
+        </is>
+      </c>
       <c r="XV9" s="6" t="n"/>
       <c r="XW9" s="6" t="n"/>
       <c r="XX9" s="6" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 04:49
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1325,7 +1325,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="24">
         <f>IF(G9="", "", RANK(G9, $G$9:$G$40))</f>
         <v/>
@@ -36146,7 +36148,11 @@
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
       <c r="AB9" s="8" t="n"/>
-      <c r="AC9" s="4" t="n"/>
+      <c r="AC9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>
       <c r="AF9" s="43" t="n"/>
@@ -48402,9 +48408,13 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n"/>
+      <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F9" s="9" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="G9" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H9" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 04:54
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1310,19 +1310,15 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>10</v>
-      </c>
+      <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Promovat</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
@@ -6893,9 +6889,7 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="E9" s="6" t="n"/>
       <c r="F9" s="8">
         <f>IF(SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9)=0, "", SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9))</f>
         <v/>
@@ -6904,14 +6898,8 @@
         <f>IF(SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9)=0, "", SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9))</f>
         <v/>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I9" s="43" t="inlineStr">
-        <is>
-          <t>28.09</t>
-        </is>
-      </c>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="43" t="n"/>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="43" t="n"/>
       <c r="L9" s="4" t="n"/>
@@ -6930,9 +6918,7 @@
       <c r="Y9" s="43" t="n"/>
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
-      <c r="AB9" s="8" t="n">
-        <v>10</v>
-      </c>
+      <c r="AB9" s="8" t="n"/>
       <c r="AC9" s="43" t="n"/>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 04:55
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1321,9 +1321,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" s="4" t="n"/>
       <c r="K9" s="24">
         <f>IF(G9="", "", RANK(G9, $G$9:$G$40))</f>
         <v/>
@@ -36193,11 +36191,7 @@
       <c r="CA9" s="4" t="n"/>
       <c r="CB9" s="43" t="n"/>
       <c r="CC9" s="6" t="n"/>
-      <c r="CD9" s="43" t="inlineStr">
-        <is>
-          <t>28.09m</t>
-        </is>
-      </c>
+      <c r="CD9" s="43" t="n"/>
       <c r="CE9" s="43" t="n"/>
       <c r="CF9" s="43" t="n"/>
       <c r="CG9" s="43" t="n"/>
@@ -48395,12 +48389,8 @@
         </is>
       </c>
       <c r="E9" s="10" t="n"/>
-      <c r="F9" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="11" t="n"/>
       <c r="H9" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:10
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1310,15 +1310,19 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="G9" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J9" s="4" t="n"/>
@@ -6887,7 +6891,9 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F9" s="8">
         <f>IF(SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9)=0, "", SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9))</f>
         <v/>
@@ -6896,8 +6902,14 @@
         <f>IF(SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9)=0, "", SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9))</f>
         <v/>
       </c>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="43" t="n"/>
+      <c r="H9" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="43" t="n"/>
       <c r="L9" s="4" t="n"/>
@@ -6916,7 +6928,9 @@
       <c r="Y9" s="43" t="n"/>
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
-      <c r="AB9" s="8" t="n"/>
+      <c r="AB9" s="8" t="n">
+        <v>10</v>
+      </c>
       <c r="AC9" s="43" t="n"/>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:11
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="24">
         <f>IF(G9="", "", RANK(G9, $G$9:$G$40))</f>
@@ -7110,7 +7110,11 @@
       <c r="GC9" s="43" t="n"/>
       <c r="GD9" s="9" t="n"/>
       <c r="GE9" s="44" t="n"/>
-      <c r="GF9" s="43" t="n"/>
+      <c r="GF9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="GG9" s="43" t="n"/>
       <c r="GH9" s="43" t="n"/>
       <c r="GI9" s="43" t="n"/>
@@ -48409,11 +48413,11 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="9" t="n"/>
       <c r="G9" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:13
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="24">
         <f>IF(G9="", "", RANK(G9, $G$9:$G$40))</f>
@@ -36152,7 +36152,11 @@
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
       <c r="AB9" s="8" t="n"/>
-      <c r="AC9" s="43" t="n"/>
+      <c r="AC9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>
       <c r="AF9" s="43" t="n"/>
@@ -48413,13 +48417,13 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:14
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -36154,7 +36154,7 @@
       <c r="AB9" s="8" t="n"/>
       <c r="AC9" s="43" t="inlineStr">
         <is>
-          <t>28.09</t>
+          <t>28.09m</t>
         </is>
       </c>
       <c r="AD9" s="43" t="n"/>
@@ -48417,10 +48417,10 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9" t="n">
         <v>2</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>1</v>
       </c>
       <c r="G9" s="11" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:55
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1311,11 +1311,11 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
@@ -1328,13 +1328,13 @@
       <c r="J9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="24">
-        <f>IF(G9="", "", RANK(G9, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L9" s="76">
-        <f>IF(K9="", "", IF(K9=1, "Premiul I", IF(K9=2, "Premiul II", IF(K9=3, "Premiul III", IF(K9&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
+      <c r="K9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="76" t="inlineStr">
+        <is>
+          <t>Premiul I</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1371,14 +1371,8 @@
         </is>
       </c>
       <c r="J10" s="4" t="n"/>
-      <c r="K10" s="24">
-        <f>IF(G10="", "", RANK(G10, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L10" s="76">
-        <f>IF(K10="", "", IF(K10=1, "Premiul I", IF(K10=2, "Premiul II", IF(K10=3, "Premiul III", IF(K10&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="76" t="n"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>6234</t>
@@ -1414,14 +1408,8 @@
         </is>
       </c>
       <c r="J11" s="4" t="n"/>
-      <c r="K11" s="24">
-        <f>IF(G11="", "", RANK(G11, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L11" s="76">
-        <f>IF(K11="", "", IF(K11=1, "Premiul I", IF(K11=2, "Premiul II", IF(K11=3, "Premiul III", IF(K11&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K11" s="24" t="n"/>
+      <c r="L11" s="76" t="n"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>9233</t>
@@ -1457,14 +1445,8 @@
         </is>
       </c>
       <c r="J12" s="4" t="n"/>
-      <c r="K12" s="24">
-        <f>IF(G12="", "", RANK(G12, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L12" s="76">
-        <f>IF(K12="", "", IF(K12=1, "Premiul I", IF(K12=2, "Premiul II", IF(K12=3, "Premiul III", IF(K12&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="76" t="n"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>9385</t>
@@ -1500,14 +1482,8 @@
         </is>
       </c>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="24">
-        <f>IF(G13="", "", RANK(G13, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L13" s="76">
-        <f>IF(K13="", "", IF(K13=1, "Premiul I", IF(K13=2, "Premiul II", IF(K13=3, "Premiul III", IF(K13&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K13" s="24" t="n"/>
+      <c r="L13" s="76" t="n"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>2681</t>
@@ -1543,14 +1519,8 @@
         </is>
       </c>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="24">
-        <f>IF(G14="", "", RANK(G14, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L14" s="76">
-        <f>IF(K14="", "", IF(K14=1, "Premiul I", IF(K14=2, "Premiul II", IF(K14=3, "Premiul III", IF(K14&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K14" s="24" t="n"/>
+      <c r="L14" s="76" t="n"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>4658</t>
@@ -1586,14 +1556,8 @@
         </is>
       </c>
       <c r="J15" s="4" t="n"/>
-      <c r="K15" s="24">
-        <f>IF(G15="", "", RANK(G15, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L15" s="76">
-        <f>IF(K15="", "", IF(K15=1, "Premiul I", IF(K15=2, "Premiul II", IF(K15=3, "Premiul III", IF(K15&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K15" s="24" t="n"/>
+      <c r="L15" s="76" t="n"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>7891</t>
@@ -1629,14 +1593,8 @@
         </is>
       </c>
       <c r="J16" s="4" t="n"/>
-      <c r="K16" s="24">
-        <f>IF(G16="", "", RANK(G16, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L16" s="76">
-        <f>IF(K16="", "", IF(K16=1, "Premiul I", IF(K16=2, "Premiul II", IF(K16=3, "Premiul III", IF(K16&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K16" s="24" t="n"/>
+      <c r="L16" s="76" t="n"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>9975</t>
@@ -1672,14 +1630,8 @@
         </is>
       </c>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="24">
-        <f>IF(G17="", "", RANK(G17, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L17" s="76">
-        <f>IF(K17="", "", IF(K17=1, "Premiul I", IF(K17=2, "Premiul II", IF(K17=3, "Premiul III", IF(K17&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K17" s="24" t="n"/>
+      <c r="L17" s="76" t="n"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>9042</t>
@@ -1715,14 +1667,8 @@
         </is>
       </c>
       <c r="J18" s="4" t="n"/>
-      <c r="K18" s="24">
-        <f>IF(G18="", "", RANK(G18, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L18" s="76">
-        <f>IF(K18="", "", IF(K18=1, "Premiul I", IF(K18=2, "Premiul II", IF(K18=3, "Premiul III", IF(K18&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K18" s="24" t="n"/>
+      <c r="L18" s="76" t="n"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>8226</t>
@@ -1758,14 +1704,8 @@
         </is>
       </c>
       <c r="J19" s="4" t="n"/>
-      <c r="K19" s="24">
-        <f>IF(G19="", "", RANK(G19, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L19" s="76">
-        <f>IF(K19="", "", IF(K19=1, "Premiul I", IF(K19=2, "Premiul II", IF(K19=3, "Premiul III", IF(K19&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K19" s="24" t="n"/>
+      <c r="L19" s="76" t="n"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>4931</t>
@@ -1801,14 +1741,8 @@
         </is>
       </c>
       <c r="J20" s="4" t="n"/>
-      <c r="K20" s="24">
-        <f>IF(G20="", "", RANK(G20, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L20" s="76">
-        <f>IF(K20="", "", IF(K20=1, "Premiul I", IF(K20=2, "Premiul II", IF(K20=3, "Premiul III", IF(K20&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K20" s="24" t="n"/>
+      <c r="L20" s="76" t="n"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>1041</t>
@@ -1844,14 +1778,8 @@
         </is>
       </c>
       <c r="J21" s="4" t="n"/>
-      <c r="K21" s="24">
-        <f>IF(G21="", "", RANK(G21, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L21" s="76">
-        <f>IF(K21="", "", IF(K21=1, "Premiul I", IF(K21=2, "Premiul II", IF(K21=3, "Premiul III", IF(K21&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K21" s="24" t="n"/>
+      <c r="L21" s="76" t="n"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>2322</t>
@@ -1887,14 +1815,8 @@
         </is>
       </c>
       <c r="J22" s="4" t="n"/>
-      <c r="K22" s="24">
-        <f>IF(G22="", "", RANK(G22, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L22" s="76">
-        <f>IF(K22="", "", IF(K22=1, "Premiul I", IF(K22=2, "Premiul II", IF(K22=3, "Premiul III", IF(K22&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K22" s="24" t="n"/>
+      <c r="L22" s="76" t="n"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>2814</t>
@@ -1930,14 +1852,8 @@
         </is>
       </c>
       <c r="J23" s="4" t="n"/>
-      <c r="K23" s="24">
-        <f>IF(G23="", "", RANK(G23, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L23" s="76">
-        <f>IF(K23="", "", IF(K23=1, "Premiul I", IF(K23=2, "Premiul II", IF(K23=3, "Premiul III", IF(K23&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K23" s="24" t="n"/>
+      <c r="L23" s="76" t="n"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>5706</t>
@@ -1973,14 +1889,8 @@
         </is>
       </c>
       <c r="J24" s="4" t="n"/>
-      <c r="K24" s="24">
-        <f>IF(G24="", "", RANK(G24, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L24" s="76">
-        <f>IF(K24="", "", IF(K24=1, "Premiul I", IF(K24=2, "Premiul II", IF(K24=3, "Premiul III", IF(K24&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K24" s="24" t="n"/>
+      <c r="L24" s="76" t="n"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>2606</t>
@@ -2016,14 +1926,8 @@
         </is>
       </c>
       <c r="J25" s="4" t="n"/>
-      <c r="K25" s="24">
-        <f>IF(G25="", "", RANK(G25, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L25" s="76">
-        <f>IF(K25="", "", IF(K25=1, "Premiul I", IF(K25=2, "Premiul II", IF(K25=3, "Premiul III", IF(K25&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K25" s="24" t="n"/>
+      <c r="L25" s="76" t="n"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>8367</t>
@@ -2059,14 +1963,8 @@
         </is>
       </c>
       <c r="J26" s="4" t="n"/>
-      <c r="K26" s="24">
-        <f>IF(G26="", "", RANK(G26, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L26" s="76">
-        <f>IF(K26="", "", IF(K26=1, "Premiul I", IF(K26=2, "Premiul II", IF(K26=3, "Premiul III", IF(K26&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K26" s="24" t="n"/>
+      <c r="L26" s="76" t="n"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>1188</t>
@@ -2102,14 +2000,8 @@
         </is>
       </c>
       <c r="J27" s="4" t="n"/>
-      <c r="K27" s="24">
-        <f>IF(G27="", "", RANK(G27, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L27" s="76">
-        <f>IF(K27="", "", IF(K27=1, "Premiul I", IF(K27=2, "Premiul II", IF(K27=3, "Premiul III", IF(K27&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K27" s="24" t="n"/>
+      <c r="L27" s="76" t="n"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>9032</t>
@@ -2145,14 +2037,8 @@
         </is>
       </c>
       <c r="J28" s="4" t="n"/>
-      <c r="K28" s="24">
-        <f>IF(G28="", "", RANK(G28, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L28" s="76">
-        <f>IF(K28="", "", IF(K28=1, "Premiul I", IF(K28=2, "Premiul II", IF(K28=3, "Premiul III", IF(K28&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K28" s="24" t="n"/>
+      <c r="L28" s="76" t="n"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>6148</t>
@@ -2188,14 +2074,8 @@
         </is>
       </c>
       <c r="J29" s="4" t="n"/>
-      <c r="K29" s="24">
-        <f>IF(G29="", "", RANK(G29, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L29" s="76">
-        <f>IF(K29="", "", IF(K29=1, "Premiul I", IF(K29=2, "Premiul II", IF(K29=3, "Premiul III", IF(K29&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K29" s="24" t="n"/>
+      <c r="L29" s="76" t="n"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>4444</t>
@@ -2231,14 +2111,8 @@
         </is>
       </c>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="24">
-        <f>IF(G30="", "", RANK(G30, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L30" s="76">
-        <f>IF(K30="", "", IF(K30=1, "Premiul I", IF(K30=2, "Premiul II", IF(K30=3, "Premiul III", IF(K30&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K30" s="24" t="n"/>
+      <c r="L30" s="76" t="n"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>7508</t>
@@ -2274,14 +2148,8 @@
         </is>
       </c>
       <c r="J31" s="4" t="n"/>
-      <c r="K31" s="24">
-        <f>IF(G31="", "", RANK(G31, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L31" s="76">
-        <f>IF(K31="", "", IF(K31=1, "Premiul I", IF(K31=2, "Premiul II", IF(K31=3, "Premiul III", IF(K31&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K31" s="24" t="n"/>
+      <c r="L31" s="76" t="n"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>5120</t>
@@ -2317,14 +2185,8 @@
         </is>
       </c>
       <c r="J32" s="4" t="n"/>
-      <c r="K32" s="24">
-        <f>IF(G32="", "", RANK(G32, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L32" s="76">
-        <f>IF(K32="", "", IF(K32=1, "Premiul I", IF(K32=2, "Premiul II", IF(K32=3, "Premiul III", IF(K32&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K32" s="24" t="n"/>
+      <c r="L32" s="76" t="n"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>6696</t>
@@ -2360,14 +2222,8 @@
         </is>
       </c>
       <c r="J33" s="4" t="n"/>
-      <c r="K33" s="24">
-        <f>IF(G33="", "", RANK(G33, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L33" s="76">
-        <f>IF(K33="", "", IF(K33=1, "Premiul I", IF(K33=2, "Premiul II", IF(K33=3, "Premiul III", IF(K33&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K33" s="24" t="n"/>
+      <c r="L33" s="76" t="n"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>6843</t>
@@ -2403,14 +2259,8 @@
         </is>
       </c>
       <c r="J34" s="4" t="n"/>
-      <c r="K34" s="24">
-        <f>IF(G34="", "", RANK(G34, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L34" s="76">
-        <f>IF(K34="", "", IF(K34=1, "Premiul I", IF(K34=2, "Premiul II", IF(K34=3, "Premiul III", IF(K34&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K34" s="24" t="n"/>
+      <c r="L34" s="76" t="n"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>7166</t>
@@ -2446,14 +2296,8 @@
         </is>
       </c>
       <c r="J35" s="4" t="n"/>
-      <c r="K35" s="24">
-        <f>IF(G35="", "", RANK(G35, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L35" s="76">
-        <f>IF(K35="", "", IF(K35=1, "Premiul I", IF(K35=2, "Premiul II", IF(K35=3, "Premiul III", IF(K35&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K35" s="24" t="n"/>
+      <c r="L35" s="76" t="n"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>9414</t>
@@ -2489,14 +2333,8 @@
         </is>
       </c>
       <c r="J36" s="4" t="n"/>
-      <c r="K36" s="24">
-        <f>IF(G36="", "", RANK(G36, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L36" s="76">
-        <f>IF(K36="", "", IF(K36=1, "Premiul I", IF(K36=2, "Premiul II", IF(K36=3, "Premiul III", IF(K36&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K36" s="24" t="n"/>
+      <c r="L36" s="76" t="n"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>2250</t>
@@ -2532,14 +2370,8 @@
         </is>
       </c>
       <c r="J37" s="4" t="n"/>
-      <c r="K37" s="24">
-        <f>IF(G37="", "", RANK(G37, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L37" s="76">
-        <f>IF(K37="", "", IF(K37=1, "Premiul I", IF(K37=2, "Premiul II", IF(K37=3, "Premiul III", IF(K37&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K37" s="24" t="n"/>
+      <c r="L37" s="76" t="n"/>
       <c r="M37" t="inlineStr">
         <is>
           <t>6577</t>
@@ -2575,14 +2407,8 @@
         </is>
       </c>
       <c r="J38" s="4" t="n"/>
-      <c r="K38" s="24">
-        <f>IF(G38="", "", RANK(G38, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L38" s="76">
-        <f>IF(K38="", "", IF(K38=1, "Premiul I", IF(K38=2, "Premiul II", IF(K38=3, "Premiul III", IF(K38&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K38" s="24" t="n"/>
+      <c r="L38" s="76" t="n"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>2469</t>
@@ -2618,14 +2444,8 @@
         </is>
       </c>
       <c r="J39" s="4" t="n"/>
-      <c r="K39" s="24">
-        <f>IF(G39="", "", RANK(G39, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L39" s="76">
-        <f>IF(K39="", "", IF(K39=1, "Premiul I", IF(K39=2, "Premiul II", IF(K39=3, "Premiul III", IF(K39&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K39" s="24" t="n"/>
+      <c r="L39" s="76" t="n"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>9815</t>
@@ -2661,14 +2481,8 @@
         </is>
       </c>
       <c r="J40" s="4" t="n"/>
-      <c r="K40" s="24">
-        <f>IF(G40="", "", RANK(G40, $G$9:$G$40))</f>
-        <v/>
-      </c>
-      <c r="L40" s="76">
-        <f>IF(K40="", "", IF(K40=1, "Premiul I", IF(K40=2, "Premiul II", IF(K40=3, "Premiul III", IF(K40&lt;=7, "Mențiune", "Membru")))))</f>
-        <v/>
-      </c>
+      <c r="K40" s="24" t="n"/>
+      <c r="L40" s="76" t="n"/>
       <c r="M40" t="inlineStr">
         <is>
           <t>5786</t>
@@ -6894,15 +6708,11 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" s="8">
-        <f>IF(SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9)=0, "", SUM(BH9,DI9,FJ9,HK9,JL9,LM9,NN9,PO9,RP9,TQ9,VR9,XS9,ZT9,ABU9))</f>
-        <v/>
-      </c>
-      <c r="G9" s="6">
-        <f>IF(SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9)=0, "", SUM(BG9,DH9,FI9,HJ9,JK9,LL9,NM9,PN9,RO9,TP9,VQ9,XR9,ZS9,ABT9))</f>
-        <v/>
+        <v>9</v>
+      </c>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
@@ -7211,8 +7021,14 @@
         <f>IF(COUNTA(IG9:JJ9)=0, "", COUNTA(IG9:JJ9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", IG9:JJ9))))</f>
         <v/>
       </c>
-      <c r="JM9" s="43" t="n"/>
-      <c r="JN9" s="43" t="n"/>
+      <c r="JM9" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="JN9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="JO9" s="43" t="n"/>
       <c r="JP9" s="43" t="n"/>
       <c r="JQ9" s="43" t="n"/>
@@ -7231,7 +7047,9 @@
       <c r="KD9" s="43" t="n"/>
       <c r="KE9" s="9" t="n"/>
       <c r="KF9" s="43" t="n"/>
-      <c r="KG9" s="44" t="n"/>
+      <c r="KG9" s="44" t="n">
+        <v>8</v>
+      </c>
       <c r="KH9" s="43" t="n"/>
       <c r="KI9" s="43" t="n"/>
       <c r="KJ9" s="43" t="n"/>
@@ -7761,14 +7579,8 @@
         </is>
       </c>
       <c r="E10" s="6" t="n"/>
-      <c r="F10" s="8">
-        <f>IF(SUM(BH10,DI10,FJ10,HK10,JL10,LM10,NN10,PO10,RP10,TQ10,VR10,XS10,ZT10,ABU10)=0, "", SUM(BH10,DI10,FJ10,HK10,JL10,LM10,NN10,PO10,RP10,TQ10,VR10,XS10,ZT10,ABU10))</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>IF(SUM(BG10,DH10,FI10,HJ10,JK10,LL10,NM10,PN10,RO10,TP10,VQ10,XR10,ZS10,ABT10)=0, "", SUM(BG10,DH10,FI10,HJ10,JK10,LL10,NM10,PN10,RO10,TP10,VQ10,XR10,ZS10,ABT10))</f>
-        <v/>
-      </c>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="6" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="43" t="n"/>
       <c r="J10" s="4" t="n"/>
@@ -8614,14 +8426,8 @@
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="8">
-        <f>IF(SUM(BH11,DI11,FJ11,HK11,JL11,LM11,NN11,PO11,RP11,TQ11,VR11,XS11,ZT11,ABU11)=0, "", SUM(BH11,DI11,FJ11,HK11,JL11,LM11,NN11,PO11,RP11,TQ11,VR11,XS11,ZT11,ABU11))</f>
-        <v/>
-      </c>
-      <c r="G11" s="6">
-        <f>IF(SUM(BG11,DH11,FI11,HJ11,JK11,LL11,NM11,PN11,RO11,TP11,VQ11,XR11,ZS11,ABT11)=0, "", SUM(BG11,DH11,FI11,HJ11,JK11,LL11,NM11,PN11,RO11,TP11,VQ11,XR11,ZS11,ABT11))</f>
-        <v/>
-      </c>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="6" t="n"/>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="43" t="n"/>
       <c r="J11" s="4" t="n"/>
@@ -9467,14 +9273,8 @@
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="8">
-        <f>IF(SUM(BH12,DI12,FJ12,HK12,JL12,LM12,NN12,PO12,RP12,TQ12,VR12,XS12,ZT12,ABU12)=0, "", SUM(BH12,DI12,FJ12,HK12,JL12,LM12,NN12,PO12,RP12,TQ12,VR12,XS12,ZT12,ABU12))</f>
-        <v/>
-      </c>
-      <c r="G12" s="6">
-        <f>IF(SUM(BG12,DH12,FI12,HJ12,JK12,LL12,NM12,PN12,RO12,TP12,VQ12,XR12,ZS12,ABT12)=0, "", SUM(BG12,DH12,FI12,HJ12,JK12,LL12,NM12,PN12,RO12,TP12,VQ12,XR12,ZS12,ABT12))</f>
-        <v/>
-      </c>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="4" t="n"/>
@@ -10320,14 +10120,8 @@
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="8">
-        <f>IF(SUM(BH13,DI13,FJ13,HK13,JL13,LM13,NN13,PO13,RP13,TQ13,VR13,XS13,ZT13,ABU13)=0, "", SUM(BH13,DI13,FJ13,HK13,JL13,LM13,NN13,PO13,RP13,TQ13,VR13,XS13,ZT13,ABU13))</f>
-        <v/>
-      </c>
-      <c r="G13" s="6">
-        <f>IF(SUM(BG13,DH13,FI13,HJ13,JK13,LL13,NM13,PN13,RO13,TP13,VQ13,XR13,ZS13,ABT13)=0, "", SUM(BG13,DH13,FI13,HJ13,JK13,LL13,NM13,PN13,RO13,TP13,VQ13,XR13,ZS13,ABT13))</f>
-        <v/>
-      </c>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="6" t="n"/>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="4" t="n"/>
@@ -11173,14 +10967,8 @@
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
-      <c r="F14" s="8">
-        <f>IF(SUM(BH14,DI14,FJ14,HK14,JL14,LM14,NN14,PO14,RP14,TQ14,VR14,XS14,ZT14,ABU14)=0, "", SUM(BH14,DI14,FJ14,HK14,JL14,LM14,NN14,PO14,RP14,TQ14,VR14,XS14,ZT14,ABU14))</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>IF(SUM(BG14,DH14,FI14,HJ14,JK14,LL14,NM14,PN14,RO14,TP14,VQ14,XR14,ZS14,ABT14)=0, "", SUM(BG14,DH14,FI14,HJ14,JK14,LL14,NM14,PN14,RO14,TP14,VQ14,XR14,ZS14,ABT14))</f>
-        <v/>
-      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="43" t="n"/>
       <c r="J14" s="4" t="n"/>
@@ -12026,14 +11814,8 @@
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
-      <c r="F15" s="8">
-        <f>IF(SUM(BH15,DI15,FJ15,HK15,JL15,LM15,NN15,PO15,RP15,TQ15,VR15,XS15,ZT15,ABU15)=0, "", SUM(BH15,DI15,FJ15,HK15,JL15,LM15,NN15,PO15,RP15,TQ15,VR15,XS15,ZT15,ABU15))</f>
-        <v/>
-      </c>
-      <c r="G15" s="6">
-        <f>IF(SUM(BG15,DH15,FI15,HJ15,JK15,LL15,NM15,PN15,RO15,TP15,VQ15,XR15,ZS15,ABT15)=0, "", SUM(BG15,DH15,FI15,HJ15,JK15,LL15,NM15,PN15,RO15,TP15,VQ15,XR15,ZS15,ABT15))</f>
-        <v/>
-      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="6" t="n"/>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="4" t="n"/>
@@ -12879,14 +12661,8 @@
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
-      <c r="F16" s="8">
-        <f>IF(SUM(BH16,DI16,FJ16,HK16,JL16,LM16,NN16,PO16,RP16,TQ16,VR16,XS16,ZT16,ABU16)=0, "", SUM(BH16,DI16,FJ16,HK16,JL16,LM16,NN16,PO16,RP16,TQ16,VR16,XS16,ZT16,ABU16))</f>
-        <v/>
-      </c>
-      <c r="G16" s="6">
-        <f>IF(SUM(BG16,DH16,FI16,HJ16,JK16,LL16,NM16,PN16,RO16,TP16,VQ16,XR16,ZS16,ABT16)=0, "", SUM(BG16,DH16,FI16,HJ16,JK16,LL16,NM16,PN16,RO16,TP16,VQ16,XR16,ZS16,ABT16))</f>
-        <v/>
-      </c>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="6" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -13732,14 +13508,8 @@
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="8">
-        <f>IF(SUM(BH17,DI17,FJ17,HK17,JL17,LM17,NN17,PO17,RP17,TQ17,VR17,XS17,ZT17,ABU17)=0, "", SUM(BH17,DI17,FJ17,HK17,JL17,LM17,NN17,PO17,RP17,TQ17,VR17,XS17,ZT17,ABU17))</f>
-        <v/>
-      </c>
-      <c r="G17" s="6">
-        <f>IF(SUM(BG17,DH17,FI17,HJ17,JK17,LL17,NM17,PN17,RO17,TP17,VQ17,XR17,ZS17,ABT17)=0, "", SUM(BG17,DH17,FI17,HJ17,JK17,LL17,NM17,PN17,RO17,TP17,VQ17,XR17,ZS17,ABT17))</f>
-        <v/>
-      </c>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="6" t="n"/>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="43" t="n"/>
       <c r="J17" s="4" t="n"/>
@@ -14585,14 +14355,8 @@
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
-      <c r="F18" s="8">
-        <f>IF(SUM(BH18,DI18,FJ18,HK18,JL18,LM18,NN18,PO18,RP18,TQ18,VR18,XS18,ZT18,ABU18)=0, "", SUM(BH18,DI18,FJ18,HK18,JL18,LM18,NN18,PO18,RP18,TQ18,VR18,XS18,ZT18,ABU18))</f>
-        <v/>
-      </c>
-      <c r="G18" s="6">
-        <f>IF(SUM(BG18,DH18,FI18,HJ18,JK18,LL18,NM18,PN18,RO18,TP18,VQ18,XR18,ZS18,ABT18)=0, "", SUM(BG18,DH18,FI18,HJ18,JK18,LL18,NM18,PN18,RO18,TP18,VQ18,XR18,ZS18,ABT18))</f>
-        <v/>
-      </c>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="43" t="n"/>
       <c r="J18" s="4" t="n"/>
@@ -15438,14 +15202,8 @@
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="8">
-        <f>IF(SUM(BH19,DI19,FJ19,HK19,JL19,LM19,NN19,PO19,RP19,TQ19,VR19,XS19,ZT19,ABU19)=0, "", SUM(BH19,DI19,FJ19,HK19,JL19,LM19,NN19,PO19,RP19,TQ19,VR19,XS19,ZT19,ABU19))</f>
-        <v/>
-      </c>
-      <c r="G19" s="6">
-        <f>IF(SUM(BG19,DH19,FI19,HJ19,JK19,LL19,NM19,PN19,RO19,TP19,VQ19,XR19,ZS19,ABT19)=0, "", SUM(BG19,DH19,FI19,HJ19,JK19,LL19,NM19,PN19,RO19,TP19,VQ19,XR19,ZS19,ABT19))</f>
-        <v/>
-      </c>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="6" t="n"/>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="43" t="n"/>
       <c r="J19" s="4" t="n"/>
@@ -16291,14 +16049,8 @@
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="8">
-        <f>IF(SUM(BH20,DI20,FJ20,HK20,JL20,LM20,NN20,PO20,RP20,TQ20,VR20,XS20,ZT20,ABU20)=0, "", SUM(BH20,DI20,FJ20,HK20,JL20,LM20,NN20,PO20,RP20,TQ20,VR20,XS20,ZT20,ABU20))</f>
-        <v/>
-      </c>
-      <c r="G20" s="6">
-        <f>IF(SUM(BG20,DH20,FI20,HJ20,JK20,LL20,NM20,PN20,RO20,TP20,VQ20,XR20,ZS20,ABT20)=0, "", SUM(BG20,DH20,FI20,HJ20,JK20,LL20,NM20,PN20,RO20,TP20,VQ20,XR20,ZS20,ABT20))</f>
-        <v/>
-      </c>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="43" t="n"/>
       <c r="J20" s="4" t="n"/>
@@ -17144,14 +16896,8 @@
         </is>
       </c>
       <c r="E21" s="6" t="n"/>
-      <c r="F21" s="8">
-        <f>IF(SUM(BH21,DI21,FJ21,HK21,JL21,LM21,NN21,PO21,RP21,TQ21,VR21,XS21,ZT21,ABU21)=0, "", SUM(BH21,DI21,FJ21,HK21,JL21,LM21,NN21,PO21,RP21,TQ21,VR21,XS21,ZT21,ABU21))</f>
-        <v/>
-      </c>
-      <c r="G21" s="6">
-        <f>IF(SUM(BG21,DH21,FI21,HJ21,JK21,LL21,NM21,PN21,RO21,TP21,VQ21,XR21,ZS21,ABT21)=0, "", SUM(BG21,DH21,FI21,HJ21,JK21,LL21,NM21,PN21,RO21,TP21,VQ21,XR21,ZS21,ABT21))</f>
-        <v/>
-      </c>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="6" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="43" t="n"/>
       <c r="J21" s="4" t="n"/>
@@ -17997,14 +17743,8 @@
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="8">
-        <f>IF(SUM(BH22,DI22,FJ22,HK22,JL22,LM22,NN22,PO22,RP22,TQ22,VR22,XS22,ZT22,ABU22)=0, "", SUM(BH22,DI22,FJ22,HK22,JL22,LM22,NN22,PO22,RP22,TQ22,VR22,XS22,ZT22,ABU22))</f>
-        <v/>
-      </c>
-      <c r="G22" s="6">
-        <f>IF(SUM(BG22,DH22,FI22,HJ22,JK22,LL22,NM22,PN22,RO22,TP22,VQ22,XR22,ZS22,ABT22)=0, "", SUM(BG22,DH22,FI22,HJ22,JK22,LL22,NM22,PN22,RO22,TP22,VQ22,XR22,ZS22,ABT22))</f>
-        <v/>
-      </c>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="6" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="43" t="n"/>
       <c r="J22" s="4" t="n"/>
@@ -18850,14 +18590,8 @@
         </is>
       </c>
       <c r="E23" s="6" t="n"/>
-      <c r="F23" s="8">
-        <f>IF(SUM(BH23,DI23,FJ23,HK23,JL23,LM23,NN23,PO23,RP23,TQ23,VR23,XS23,ZT23,ABU23)=0, "", SUM(BH23,DI23,FJ23,HK23,JL23,LM23,NN23,PO23,RP23,TQ23,VR23,XS23,ZT23,ABU23))</f>
-        <v/>
-      </c>
-      <c r="G23" s="6">
-        <f>IF(SUM(BG23,DH23,FI23,HJ23,JK23,LL23,NM23,PN23,RO23,TP23,VQ23,XR23,ZS23,ABT23)=0, "", SUM(BG23,DH23,FI23,HJ23,JK23,LL23,NM23,PN23,RO23,TP23,VQ23,XR23,ZS23,ABT23))</f>
-        <v/>
-      </c>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="6" t="n"/>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
       <c r="J23" s="4" t="n"/>
@@ -19703,14 +19437,8 @@
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
-      <c r="F24" s="8">
-        <f>IF(SUM(BH24,DI24,FJ24,HK24,JL24,LM24,NN24,PO24,RP24,TQ24,VR24,XS24,ZT24,ABU24)=0, "", SUM(BH24,DI24,FJ24,HK24,JL24,LM24,NN24,PO24,RP24,TQ24,VR24,XS24,ZT24,ABU24))</f>
-        <v/>
-      </c>
-      <c r="G24" s="6">
-        <f>IF(SUM(BG24,DH24,FI24,HJ24,JK24,LL24,NM24,PN24,RO24,TP24,VQ24,XR24,ZS24,ABT24)=0, "", SUM(BG24,DH24,FI24,HJ24,JK24,LL24,NM24,PN24,RO24,TP24,VQ24,XR24,ZS24,ABT24))</f>
-        <v/>
-      </c>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="6" t="n"/>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="43" t="n"/>
       <c r="J24" s="4" t="n"/>
@@ -20556,14 +20284,8 @@
         </is>
       </c>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="8">
-        <f>IF(SUM(BH25,DI25,FJ25,HK25,JL25,LM25,NN25,PO25,RP25,TQ25,VR25,XS25,ZT25,ABU25)=0, "", SUM(BH25,DI25,FJ25,HK25,JL25,LM25,NN25,PO25,RP25,TQ25,VR25,XS25,ZT25,ABU25))</f>
-        <v/>
-      </c>
-      <c r="G25" s="6">
-        <f>IF(SUM(BG25,DH25,FI25,HJ25,JK25,LL25,NM25,PN25,RO25,TP25,VQ25,XR25,ZS25,ABT25)=0, "", SUM(BG25,DH25,FI25,HJ25,JK25,LL25,NM25,PN25,RO25,TP25,VQ25,XR25,ZS25,ABT25))</f>
-        <v/>
-      </c>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="6" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="43" t="n"/>
       <c r="J25" s="4" t="n"/>
@@ -21409,14 +21131,8 @@
         </is>
       </c>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8">
-        <f>IF(SUM(BH26,DI26,FJ26,HK26,JL26,LM26,NN26,PO26,RP26,TQ26,VR26,XS26,ZT26,ABU26)=0, "", SUM(BH26,DI26,FJ26,HK26,JL26,LM26,NN26,PO26,RP26,TQ26,VR26,XS26,ZT26,ABU26))</f>
-        <v/>
-      </c>
-      <c r="G26" s="6">
-        <f>IF(SUM(BG26,DH26,FI26,HJ26,JK26,LL26,NM26,PN26,RO26,TP26,VQ26,XR26,ZS26,ABT26)=0, "", SUM(BG26,DH26,FI26,HJ26,JK26,LL26,NM26,PN26,RO26,TP26,VQ26,XR26,ZS26,ABT26))</f>
-        <v/>
-      </c>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="6" t="n"/>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="43" t="n"/>
       <c r="J26" s="4" t="n"/>
@@ -22262,14 +21978,8 @@
         </is>
       </c>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="8">
-        <f>IF(SUM(BH27,DI27,FJ27,HK27,JL27,LM27,NN27,PO27,RP27,TQ27,VR27,XS27,ZT27,ABU27)=0, "", SUM(BH27,DI27,FJ27,HK27,JL27,LM27,NN27,PO27,RP27,TQ27,VR27,XS27,ZT27,ABU27))</f>
-        <v/>
-      </c>
-      <c r="G27" s="6">
-        <f>IF(SUM(BG27,DH27,FI27,HJ27,JK27,LL27,NM27,PN27,RO27,TP27,VQ27,XR27,ZS27,ABT27)=0, "", SUM(BG27,DH27,FI27,HJ27,JK27,LL27,NM27,PN27,RO27,TP27,VQ27,XR27,ZS27,ABT27))</f>
-        <v/>
-      </c>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="6" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="43" t="n"/>
       <c r="J27" s="4" t="n"/>
@@ -23115,14 +22825,8 @@
         </is>
       </c>
       <c r="E28" s="6" t="n"/>
-      <c r="F28" s="8">
-        <f>IF(SUM(BH28,DI28,FJ28,HK28,JL28,LM28,NN28,PO28,RP28,TQ28,VR28,XS28,ZT28,ABU28)=0, "", SUM(BH28,DI28,FJ28,HK28,JL28,LM28,NN28,PO28,RP28,TQ28,VR28,XS28,ZT28,ABU28))</f>
-        <v/>
-      </c>
-      <c r="G28" s="6">
-        <f>IF(SUM(BG28,DH28,FI28,HJ28,JK28,LL28,NM28,PN28,RO28,TP28,VQ28,XR28,ZS28,ABT28)=0, "", SUM(BG28,DH28,FI28,HJ28,JK28,LL28,NM28,PN28,RO28,TP28,VQ28,XR28,ZS28,ABT28))</f>
-        <v/>
-      </c>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="6" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="43" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -23968,14 +23672,8 @@
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="8">
-        <f>IF(SUM(BH29,DI29,FJ29,HK29,JL29,LM29,NN29,PO29,RP29,TQ29,VR29,XS29,ZT29,ABU29)=0, "", SUM(BH29,DI29,FJ29,HK29,JL29,LM29,NN29,PO29,RP29,TQ29,VR29,XS29,ZT29,ABU29))</f>
-        <v/>
-      </c>
-      <c r="G29" s="6">
-        <f>IF(SUM(BG29,DH29,FI29,HJ29,JK29,LL29,NM29,PN29,RO29,TP29,VQ29,XR29,ZS29,ABT29)=0, "", SUM(BG29,DH29,FI29,HJ29,JK29,LL29,NM29,PN29,RO29,TP29,VQ29,XR29,ZS29,ABT29))</f>
-        <v/>
-      </c>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="6" t="n"/>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="43" t="n"/>
       <c r="J29" s="4" t="n"/>
@@ -24821,14 +24519,8 @@
         </is>
       </c>
       <c r="E30" s="6" t="n"/>
-      <c r="F30" s="8">
-        <f>IF(SUM(BH30,DI30,FJ30,HK30,JL30,LM30,NN30,PO30,RP30,TQ30,VR30,XS30,ZT30,ABU30)=0, "", SUM(BH30,DI30,FJ30,HK30,JL30,LM30,NN30,PO30,RP30,TQ30,VR30,XS30,ZT30,ABU30))</f>
-        <v/>
-      </c>
-      <c r="G30" s="6">
-        <f>IF(SUM(BG30,DH30,FI30,HJ30,JK30,LL30,NM30,PN30,RO30,TP30,VQ30,XR30,ZS30,ABT30)=0, "", SUM(BG30,DH30,FI30,HJ30,JK30,LL30,NM30,PN30,RO30,TP30,VQ30,XR30,ZS30,ABT30))</f>
-        <v/>
-      </c>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="43" t="n"/>
       <c r="J30" s="4" t="n"/>
@@ -25674,14 +25366,8 @@
         </is>
       </c>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="8">
-        <f>IF(SUM(BH31,DI31,FJ31,HK31,JL31,LM31,NN31,PO31,RP31,TQ31,VR31,XS31,ZT31,ABU31)=0, "", SUM(BH31,DI31,FJ31,HK31,JL31,LM31,NN31,PO31,RP31,TQ31,VR31,XS31,ZT31,ABU31))</f>
-        <v/>
-      </c>
-      <c r="G31" s="6">
-        <f>IF(SUM(BG31,DH31,FI31,HJ31,JK31,LL31,NM31,PN31,RO31,TP31,VQ31,XR31,ZS31,ABT31)=0, "", SUM(BG31,DH31,FI31,HJ31,JK31,LL31,NM31,PN31,RO31,TP31,VQ31,XR31,ZS31,ABT31))</f>
-        <v/>
-      </c>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="43" t="n"/>
       <c r="J31" s="4" t="n"/>
@@ -26527,14 +26213,8 @@
         </is>
       </c>
       <c r="E32" s="6" t="n"/>
-      <c r="F32" s="8">
-        <f>IF(SUM(BH32,DI32,FJ32,HK32,JL32,LM32,NN32,PO32,RP32,TQ32,VR32,XS32,ZT32,ABU32)=0, "", SUM(BH32,DI32,FJ32,HK32,JL32,LM32,NN32,PO32,RP32,TQ32,VR32,XS32,ZT32,ABU32))</f>
-        <v/>
-      </c>
-      <c r="G32" s="6">
-        <f>IF(SUM(BG32,DH32,FI32,HJ32,JK32,LL32,NM32,PN32,RO32,TP32,VQ32,XR32,ZS32,ABT32)=0, "", SUM(BG32,DH32,FI32,HJ32,JK32,LL32,NM32,PN32,RO32,TP32,VQ32,XR32,ZS32,ABT32))</f>
-        <v/>
-      </c>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="6" t="n"/>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="43" t="n"/>
       <c r="J32" s="4" t="n"/>
@@ -27380,14 +27060,8 @@
         </is>
       </c>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="8">
-        <f>IF(SUM(BH33,DI33,FJ33,HK33,JL33,LM33,NN33,PO33,RP33,TQ33,VR33,XS33,ZT33,ABU33)=0, "", SUM(BH33,DI33,FJ33,HK33,JL33,LM33,NN33,PO33,RP33,TQ33,VR33,XS33,ZT33,ABU33))</f>
-        <v/>
-      </c>
-      <c r="G33" s="6">
-        <f>IF(SUM(BG33,DH33,FI33,HJ33,JK33,LL33,NM33,PN33,RO33,TP33,VQ33,XR33,ZS33,ABT33)=0, "", SUM(BG33,DH33,FI33,HJ33,JK33,LL33,NM33,PN33,RO33,TP33,VQ33,XR33,ZS33,ABT33))</f>
-        <v/>
-      </c>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="6" t="n"/>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="43" t="n"/>
       <c r="J33" s="4" t="n"/>
@@ -28233,14 +27907,8 @@
         </is>
       </c>
       <c r="E34" s="6" t="n"/>
-      <c r="F34" s="8">
-        <f>IF(SUM(BH34,DI34,FJ34,HK34,JL34,LM34,NN34,PO34,RP34,TQ34,VR34,XS34,ZT34,ABU34)=0, "", SUM(BH34,DI34,FJ34,HK34,JL34,LM34,NN34,PO34,RP34,TQ34,VR34,XS34,ZT34,ABU34))</f>
-        <v/>
-      </c>
-      <c r="G34" s="6">
-        <f>IF(SUM(BG34,DH34,FI34,HJ34,JK34,LL34,NM34,PN34,RO34,TP34,VQ34,XR34,ZS34,ABT34)=0, "", SUM(BG34,DH34,FI34,HJ34,JK34,LL34,NM34,PN34,RO34,TP34,VQ34,XR34,ZS34,ABT34))</f>
-        <v/>
-      </c>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="6" t="n"/>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="43" t="n"/>
       <c r="J34" s="4" t="n"/>
@@ -29086,14 +28754,8 @@
         </is>
       </c>
       <c r="E35" s="6" t="n"/>
-      <c r="F35" s="8">
-        <f>IF(SUM(BH35,DI35,FJ35,HK35,JL35,LM35,NN35,PO35,RP35,TQ35,VR35,XS35,ZT35,ABU35)=0, "", SUM(BH35,DI35,FJ35,HK35,JL35,LM35,NN35,PO35,RP35,TQ35,VR35,XS35,ZT35,ABU35))</f>
-        <v/>
-      </c>
-      <c r="G35" s="6">
-        <f>IF(SUM(BG35,DH35,FI35,HJ35,JK35,LL35,NM35,PN35,RO35,TP35,VQ35,XR35,ZS35,ABT35)=0, "", SUM(BG35,DH35,FI35,HJ35,JK35,LL35,NM35,PN35,RO35,TP35,VQ35,XR35,ZS35,ABT35))</f>
-        <v/>
-      </c>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="6" t="n"/>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="43" t="n"/>
       <c r="J35" s="4" t="n"/>
@@ -29939,14 +29601,8 @@
         </is>
       </c>
       <c r="E36" s="6" t="n"/>
-      <c r="F36" s="8">
-        <f>IF(SUM(BH36,DI36,FJ36,HK36,JL36,LM36,NN36,PO36,RP36,TQ36,VR36,XS36,ZT36,ABU36)=0, "", SUM(BH36,DI36,FJ36,HK36,JL36,LM36,NN36,PO36,RP36,TQ36,VR36,XS36,ZT36,ABU36))</f>
-        <v/>
-      </c>
-      <c r="G36" s="6">
-        <f>IF(SUM(BG36,DH36,FI36,HJ36,JK36,LL36,NM36,PN36,RO36,TP36,VQ36,XR36,ZS36,ABT36)=0, "", SUM(BG36,DH36,FI36,HJ36,JK36,LL36,NM36,PN36,RO36,TP36,VQ36,XR36,ZS36,ABT36))</f>
-        <v/>
-      </c>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="6" t="n"/>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="43" t="n"/>
       <c r="J36" s="4" t="n"/>
@@ -30792,14 +30448,8 @@
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="8">
-        <f>IF(SUM(BH37,DI37,FJ37,HK37,JL37,LM37,NN37,PO37,RP37,TQ37,VR37,XS37,ZT37,ABU37)=0, "", SUM(BH37,DI37,FJ37,HK37,JL37,LM37,NN37,PO37,RP37,TQ37,VR37,XS37,ZT37,ABU37))</f>
-        <v/>
-      </c>
-      <c r="G37" s="6">
-        <f>IF(SUM(BG37,DH37,FI37,HJ37,JK37,LL37,NM37,PN37,RO37,TP37,VQ37,XR37,ZS37,ABT37)=0, "", SUM(BG37,DH37,FI37,HJ37,JK37,LL37,NM37,PN37,RO37,TP37,VQ37,XR37,ZS37,ABT37))</f>
-        <v/>
-      </c>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="6" t="n"/>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="43" t="n"/>
       <c r="J37" s="4" t="n"/>
@@ -31645,14 +31295,8 @@
         </is>
       </c>
       <c r="E38" s="6" t="n"/>
-      <c r="F38" s="8">
-        <f>IF(SUM(BH38,DI38,FJ38,HK38,JL38,LM38,NN38,PO38,RP38,TQ38,VR38,XS38,ZT38,ABU38)=0, "", SUM(BH38,DI38,FJ38,HK38,JL38,LM38,NN38,PO38,RP38,TQ38,VR38,XS38,ZT38,ABU38))</f>
-        <v/>
-      </c>
-      <c r="G38" s="6">
-        <f>IF(SUM(BG38,DH38,FI38,HJ38,JK38,LL38,NM38,PN38,RO38,TP38,VQ38,XR38,ZS38,ABT38)=0, "", SUM(BG38,DH38,FI38,HJ38,JK38,LL38,NM38,PN38,RO38,TP38,VQ38,XR38,ZS38,ABT38))</f>
-        <v/>
-      </c>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="6" t="n"/>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="43" t="n"/>
       <c r="J38" s="4" t="n"/>
@@ -32498,14 +32142,8 @@
         </is>
       </c>
       <c r="E39" s="6" t="n"/>
-      <c r="F39" s="8">
-        <f>IF(SUM(BH39,DI39,FJ39,HK39,JL39,LM39,NN39,PO39,RP39,TQ39,VR39,XS39,ZT39,ABU39)=0, "", SUM(BH39,DI39,FJ39,HK39,JL39,LM39,NN39,PO39,RP39,TQ39,VR39,XS39,ZT39,ABU39))</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>IF(SUM(BG39,DH39,FI39,HJ39,JK39,LL39,NM39,PN39,RO39,TP39,VQ39,XR39,ZS39,ABT39)=0, "", SUM(BG39,DH39,FI39,HJ39,JK39,LL39,NM39,PN39,RO39,TP39,VQ39,XR39,ZS39,ABT39))</f>
-        <v/>
-      </c>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="6" t="n"/>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="43" t="n"/>
       <c r="J39" s="4" t="n"/>
@@ -33351,14 +32989,8 @@
         </is>
       </c>
       <c r="E40" s="6" t="n"/>
-      <c r="F40" s="8">
-        <f>IF(SUM(BH40,DI40,FJ40,HK40,JL40,LM40,NN40,PO40,RP40,TQ40,VR40,XS40,ZT40,ABU40)=0, "", SUM(BH40,DI40,FJ40,HK40,JL40,LM40,NN40,PO40,RP40,TQ40,VR40,XS40,ZT40,ABU40))</f>
-        <v/>
-      </c>
-      <c r="G40" s="6">
-        <f>IF(SUM(BG40,DH40,FI40,HJ40,JK40,LL40,NM40,PN40,RO40,TP40,VQ40,XR40,ZS40,ABT40)=0, "", SUM(BG40,DH40,FI40,HJ40,JK40,LL40,NM40,PN40,RO40,TP40,VQ40,XR40,ZS40,ABT40))</f>
-        <v/>
-      </c>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="6" t="n"/>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
       <c r="J40" s="4" t="n"/>
@@ -36123,13 +35755,11 @@
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="8">
-        <f>IF(SUM(BH9,DI9,FJ9,HK9,JL9,LM9)=0, "", SUM(BH9,DI9,FJ9,HK9,JL9,LM9))</f>
-        <v/>
-      </c>
-      <c r="G9" s="6">
-        <f>IF(SUM(BG9,DH9,FI9,HJ9,JK9,LL9)=0, "", SUM(BG9,DH9,FI9,HJ9,JK9,LL9))</f>
-        <v/>
+      <c r="F9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="43" t="n"/>
@@ -36512,14 +36142,8 @@
         </is>
       </c>
       <c r="E10" s="6" t="n"/>
-      <c r="F10" s="8">
-        <f>IF(SUM(BH10,DI10,FJ10,HK10,JL10,LM10)=0, "", SUM(BH10,DI10,FJ10,HK10,JL10,LM10))</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>IF(SUM(BG10,DH10,FI10,HJ10,JK10,LL10)=0, "", SUM(BG10,DH10,FI10,HJ10,JK10,LL10))</f>
-        <v/>
-      </c>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="6" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="43" t="n"/>
       <c r="J10" s="4" t="n"/>
@@ -36893,14 +36517,8 @@
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="8">
-        <f>IF(SUM(BH11,DI11,FJ11,HK11,JL11,LM11)=0, "", SUM(BH11,DI11,FJ11,HK11,JL11,LM11))</f>
-        <v/>
-      </c>
-      <c r="G11" s="6">
-        <f>IF(SUM(BG11,DH11,FI11,HJ11,JK11,LL11)=0, "", SUM(BG11,DH11,FI11,HJ11,JK11,LL11))</f>
-        <v/>
-      </c>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="6" t="n"/>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="43" t="n"/>
       <c r="J11" s="4" t="n"/>
@@ -37274,14 +36892,8 @@
         </is>
       </c>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="8">
-        <f>IF(SUM(BH12,DI12,FJ12,HK12,JL12,LM12)=0, "", SUM(BH12,DI12,FJ12,HK12,JL12,LM12))</f>
-        <v/>
-      </c>
-      <c r="G12" s="6">
-        <f>IF(SUM(BG12,DH12,FI12,HJ12,JK12,LL12)=0, "", SUM(BG12,DH12,FI12,HJ12,JK12,LL12))</f>
-        <v/>
-      </c>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="4" t="n"/>
@@ -37655,14 +37267,8 @@
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
-      <c r="F13" s="8">
-        <f>IF(SUM(BH13,DI13,FJ13,HK13,JL13,LM13)=0, "", SUM(BH13,DI13,FJ13,HK13,JL13,LM13))</f>
-        <v/>
-      </c>
-      <c r="G13" s="6">
-        <f>IF(SUM(BG13,DH13,FI13,HJ13,JK13,LL13)=0, "", SUM(BG13,DH13,FI13,HJ13,JK13,LL13))</f>
-        <v/>
-      </c>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="6" t="n"/>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="4" t="n"/>
@@ -38036,14 +37642,8 @@
         </is>
       </c>
       <c r="E14" s="6" t="n"/>
-      <c r="F14" s="8">
-        <f>IF(SUM(BH14,DI14,FJ14,HK14,JL14,LM14)=0, "", SUM(BH14,DI14,FJ14,HK14,JL14,LM14))</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>IF(SUM(BG14,DH14,FI14,HJ14,JK14,LL14)=0, "", SUM(BG14,DH14,FI14,HJ14,JK14,LL14))</f>
-        <v/>
-      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="43" t="n"/>
       <c r="J14" s="4" t="n"/>
@@ -38417,14 +38017,8 @@
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
-      <c r="F15" s="8">
-        <f>IF(SUM(BH15,DI15,FJ15,HK15,JL15,LM15)=0, "", SUM(BH15,DI15,FJ15,HK15,JL15,LM15))</f>
-        <v/>
-      </c>
-      <c r="G15" s="6">
-        <f>IF(SUM(BG15,DH15,FI15,HJ15,JK15,LL15)=0, "", SUM(BG15,DH15,FI15,HJ15,JK15,LL15))</f>
-        <v/>
-      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="6" t="n"/>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="4" t="n"/>
@@ -38798,14 +38392,8 @@
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
-      <c r="F16" s="8">
-        <f>IF(SUM(BH16,DI16,FJ16,HK16,JL16,LM16)=0, "", SUM(BH16,DI16,FJ16,HK16,JL16,LM16))</f>
-        <v/>
-      </c>
-      <c r="G16" s="6">
-        <f>IF(SUM(BG16,DH16,FI16,HJ16,JK16,LL16)=0, "", SUM(BG16,DH16,FI16,HJ16,JK16,LL16))</f>
-        <v/>
-      </c>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="6" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -39179,14 +38767,8 @@
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
-      <c r="F17" s="8">
-        <f>IF(SUM(BH17,DI17,FJ17,HK17,JL17,LM17)=0, "", SUM(BH17,DI17,FJ17,HK17,JL17,LM17))</f>
-        <v/>
-      </c>
-      <c r="G17" s="6">
-        <f>IF(SUM(BG17,DH17,FI17,HJ17,JK17,LL17)=0, "", SUM(BG17,DH17,FI17,HJ17,JK17,LL17))</f>
-        <v/>
-      </c>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="6" t="n"/>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="43" t="n"/>
       <c r="J17" s="4" t="n"/>
@@ -39560,14 +39142,8 @@
         </is>
       </c>
       <c r="E18" s="6" t="n"/>
-      <c r="F18" s="8">
-        <f>IF(SUM(BH18,DI18,FJ18,HK18,JL18,LM18)=0, "", SUM(BH18,DI18,FJ18,HK18,JL18,LM18))</f>
-        <v/>
-      </c>
-      <c r="G18" s="6">
-        <f>IF(SUM(BG18,DH18,FI18,HJ18,JK18,LL18)=0, "", SUM(BG18,DH18,FI18,HJ18,JK18,LL18))</f>
-        <v/>
-      </c>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="43" t="n"/>
       <c r="J18" s="4" t="n"/>
@@ -39941,14 +39517,8 @@
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="8">
-        <f>IF(SUM(BH19,DI19,FJ19,HK19,JL19,LM19)=0, "", SUM(BH19,DI19,FJ19,HK19,JL19,LM19))</f>
-        <v/>
-      </c>
-      <c r="G19" s="6">
-        <f>IF(SUM(BG19,DH19,FI19,HJ19,JK19,LL19)=0, "", SUM(BG19,DH19,FI19,HJ19,JK19,LL19))</f>
-        <v/>
-      </c>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="6" t="n"/>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="43" t="n"/>
       <c r="J19" s="4" t="n"/>
@@ -40322,14 +39892,8 @@
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="8">
-        <f>IF(SUM(BH20,DI20,FJ20,HK20,JL20,LM20)=0, "", SUM(BH20,DI20,FJ20,HK20,JL20,LM20))</f>
-        <v/>
-      </c>
-      <c r="G20" s="6">
-        <f>IF(SUM(BG20,DH20,FI20,HJ20,JK20,LL20)=0, "", SUM(BG20,DH20,FI20,HJ20,JK20,LL20))</f>
-        <v/>
-      </c>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="43" t="n"/>
       <c r="J20" s="4" t="n"/>
@@ -40703,14 +40267,8 @@
         </is>
       </c>
       <c r="E21" s="6" t="n"/>
-      <c r="F21" s="8">
-        <f>IF(SUM(BH21,DI21,FJ21,HK21,JL21,LM21)=0, "", SUM(BH21,DI21,FJ21,HK21,JL21,LM21))</f>
-        <v/>
-      </c>
-      <c r="G21" s="6">
-        <f>IF(SUM(BG21,DH21,FI21,HJ21,JK21,LL21)=0, "", SUM(BG21,DH21,FI21,HJ21,JK21,LL21))</f>
-        <v/>
-      </c>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="6" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="43" t="n"/>
       <c r="J21" s="4" t="n"/>
@@ -41084,14 +40642,8 @@
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="8">
-        <f>IF(SUM(BH22,DI22,FJ22,HK22,JL22,LM22)=0, "", SUM(BH22,DI22,FJ22,HK22,JL22,LM22))</f>
-        <v/>
-      </c>
-      <c r="G22" s="6">
-        <f>IF(SUM(BG22,DH22,FI22,HJ22,JK22,LL22)=0, "", SUM(BG22,DH22,FI22,HJ22,JK22,LL22))</f>
-        <v/>
-      </c>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="6" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="43" t="n"/>
       <c r="J22" s="4" t="n"/>
@@ -41465,14 +41017,8 @@
         </is>
       </c>
       <c r="E23" s="6" t="n"/>
-      <c r="F23" s="8">
-        <f>IF(SUM(BH23,DI23,FJ23,HK23,JL23,LM23)=0, "", SUM(BH23,DI23,FJ23,HK23,JL23,LM23))</f>
-        <v/>
-      </c>
-      <c r="G23" s="6">
-        <f>IF(SUM(BG23,DH23,FI23,HJ23,JK23,LL23)=0, "", SUM(BG23,DH23,FI23,HJ23,JK23,LL23))</f>
-        <v/>
-      </c>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="6" t="n"/>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
       <c r="J23" s="4" t="n"/>
@@ -41846,14 +41392,8 @@
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
-      <c r="F24" s="8">
-        <f>IF(SUM(BH24,DI24,FJ24,HK24,JL24,LM24)=0, "", SUM(BH24,DI24,FJ24,HK24,JL24,LM24))</f>
-        <v/>
-      </c>
-      <c r="G24" s="6">
-        <f>IF(SUM(BG24,DH24,FI24,HJ24,JK24,LL24)=0, "", SUM(BG24,DH24,FI24,HJ24,JK24,LL24))</f>
-        <v/>
-      </c>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="6" t="n"/>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="43" t="n"/>
       <c r="J24" s="4" t="n"/>
@@ -42227,14 +41767,8 @@
         </is>
       </c>
       <c r="E25" s="6" t="n"/>
-      <c r="F25" s="8">
-        <f>IF(SUM(BH25,DI25,FJ25,HK25,JL25,LM25)=0, "", SUM(BH25,DI25,FJ25,HK25,JL25,LM25))</f>
-        <v/>
-      </c>
-      <c r="G25" s="6">
-        <f>IF(SUM(BG25,DH25,FI25,HJ25,JK25,LL25)=0, "", SUM(BG25,DH25,FI25,HJ25,JK25,LL25))</f>
-        <v/>
-      </c>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="6" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="43" t="n"/>
       <c r="J25" s="4" t="n"/>
@@ -42608,14 +42142,8 @@
         </is>
       </c>
       <c r="E26" s="6" t="n"/>
-      <c r="F26" s="8">
-        <f>IF(SUM(BH26,DI26,FJ26,HK26,JL26,LM26)=0, "", SUM(BH26,DI26,FJ26,HK26,JL26,LM26))</f>
-        <v/>
-      </c>
-      <c r="G26" s="6">
-        <f>IF(SUM(BG26,DH26,FI26,HJ26,JK26,LL26)=0, "", SUM(BG26,DH26,FI26,HJ26,JK26,LL26))</f>
-        <v/>
-      </c>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="6" t="n"/>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="43" t="n"/>
       <c r="J26" s="4" t="n"/>
@@ -42989,14 +42517,8 @@
         </is>
       </c>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="8">
-        <f>IF(SUM(BH27,DI27,FJ27,HK27,JL27,LM27)=0, "", SUM(BH27,DI27,FJ27,HK27,JL27,LM27))</f>
-        <v/>
-      </c>
-      <c r="G27" s="6">
-        <f>IF(SUM(BG27,DH27,FI27,HJ27,JK27,LL27)=0, "", SUM(BG27,DH27,FI27,HJ27,JK27,LL27))</f>
-        <v/>
-      </c>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="6" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="43" t="n"/>
       <c r="J27" s="4" t="n"/>
@@ -43370,14 +42892,8 @@
         </is>
       </c>
       <c r="E28" s="6" t="n"/>
-      <c r="F28" s="8">
-        <f>IF(SUM(BH28,DI28,FJ28,HK28,JL28,LM28)=0, "", SUM(BH28,DI28,FJ28,HK28,JL28,LM28))</f>
-        <v/>
-      </c>
-      <c r="G28" s="6">
-        <f>IF(SUM(BG28,DH28,FI28,HJ28,JK28,LL28)=0, "", SUM(BG28,DH28,FI28,HJ28,JK28,LL28))</f>
-        <v/>
-      </c>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="6" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="43" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -43751,14 +43267,8 @@
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="8">
-        <f>IF(SUM(BH29,DI29,FJ29,HK29,JL29,LM29)=0, "", SUM(BH29,DI29,FJ29,HK29,JL29,LM29))</f>
-        <v/>
-      </c>
-      <c r="G29" s="6">
-        <f>IF(SUM(BG29,DH29,FI29,HJ29,JK29,LL29)=0, "", SUM(BG29,DH29,FI29,HJ29,JK29,LL29))</f>
-        <v/>
-      </c>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="6" t="n"/>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="43" t="n"/>
       <c r="J29" s="4" t="n"/>
@@ -44132,14 +43642,8 @@
         </is>
       </c>
       <c r="E30" s="6" t="n"/>
-      <c r="F30" s="8">
-        <f>IF(SUM(BH30,DI30,FJ30,HK30,JL30,LM30)=0, "", SUM(BH30,DI30,FJ30,HK30,JL30,LM30))</f>
-        <v/>
-      </c>
-      <c r="G30" s="6">
-        <f>IF(SUM(BG30,DH30,FI30,HJ30,JK30,LL30)=0, "", SUM(BG30,DH30,FI30,HJ30,JK30,LL30))</f>
-        <v/>
-      </c>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="43" t="n"/>
       <c r="J30" s="4" t="n"/>
@@ -44513,14 +44017,8 @@
         </is>
       </c>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="8">
-        <f>IF(SUM(BH31,DI31,FJ31,HK31,JL31,LM31)=0, "", SUM(BH31,DI31,FJ31,HK31,JL31,LM31))</f>
-        <v/>
-      </c>
-      <c r="G31" s="6">
-        <f>IF(SUM(BG31,DH31,FI31,HJ31,JK31,LL31)=0, "", SUM(BG31,DH31,FI31,HJ31,JK31,LL31))</f>
-        <v/>
-      </c>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="43" t="n"/>
       <c r="J31" s="4" t="n"/>
@@ -44894,14 +44392,8 @@
         </is>
       </c>
       <c r="E32" s="6" t="n"/>
-      <c r="F32" s="8">
-        <f>IF(SUM(BH32,DI32,FJ32,HK32,JL32,LM32)=0, "", SUM(BH32,DI32,FJ32,HK32,JL32,LM32))</f>
-        <v/>
-      </c>
-      <c r="G32" s="6">
-        <f>IF(SUM(BG32,DH32,FI32,HJ32,JK32,LL32)=0, "", SUM(BG32,DH32,FI32,HJ32,JK32,LL32))</f>
-        <v/>
-      </c>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="6" t="n"/>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="43" t="n"/>
       <c r="J32" s="4" t="n"/>
@@ -45275,14 +44767,8 @@
         </is>
       </c>
       <c r="E33" s="6" t="n"/>
-      <c r="F33" s="8">
-        <f>IF(SUM(BH33,DI33,FJ33,HK33,JL33,LM33)=0, "", SUM(BH33,DI33,FJ33,HK33,JL33,LM33))</f>
-        <v/>
-      </c>
-      <c r="G33" s="6">
-        <f>IF(SUM(BG33,DH33,FI33,HJ33,JK33,LL33)=0, "", SUM(BG33,DH33,FI33,HJ33,JK33,LL33))</f>
-        <v/>
-      </c>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="6" t="n"/>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="43" t="n"/>
       <c r="J33" s="4" t="n"/>
@@ -45656,14 +45142,8 @@
         </is>
       </c>
       <c r="E34" s="6" t="n"/>
-      <c r="F34" s="8">
-        <f>IF(SUM(BH34,DI34,FJ34,HK34,JL34,LM34)=0, "", SUM(BH34,DI34,FJ34,HK34,JL34,LM34))</f>
-        <v/>
-      </c>
-      <c r="G34" s="6">
-        <f>IF(SUM(BG34,DH34,FI34,HJ34,JK34,LL34)=0, "", SUM(BG34,DH34,FI34,HJ34,JK34,LL34))</f>
-        <v/>
-      </c>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="6" t="n"/>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="43" t="n"/>
       <c r="J34" s="4" t="n"/>
@@ -46037,14 +45517,8 @@
         </is>
       </c>
       <c r="E35" s="6" t="n"/>
-      <c r="F35" s="8">
-        <f>IF(SUM(BH35,DI35,FJ35,HK35,JL35,LM35)=0, "", SUM(BH35,DI35,FJ35,HK35,JL35,LM35))</f>
-        <v/>
-      </c>
-      <c r="G35" s="6">
-        <f>IF(SUM(BG35,DH35,FI35,HJ35,JK35,LL35)=0, "", SUM(BG35,DH35,FI35,HJ35,JK35,LL35))</f>
-        <v/>
-      </c>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="6" t="n"/>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="43" t="n"/>
       <c r="J35" s="4" t="n"/>
@@ -46418,14 +45892,8 @@
         </is>
       </c>
       <c r="E36" s="6" t="n"/>
-      <c r="F36" s="8">
-        <f>IF(SUM(BH36,DI36,FJ36,HK36,JL36,LM36)=0, "", SUM(BH36,DI36,FJ36,HK36,JL36,LM36))</f>
-        <v/>
-      </c>
-      <c r="G36" s="6">
-        <f>IF(SUM(BG36,DH36,FI36,HJ36,JK36,LL36)=0, "", SUM(BG36,DH36,FI36,HJ36,JK36,LL36))</f>
-        <v/>
-      </c>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="6" t="n"/>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="43" t="n"/>
       <c r="J36" s="4" t="n"/>
@@ -46799,14 +46267,8 @@
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="8">
-        <f>IF(SUM(BH37,DI37,FJ37,HK37,JL37,LM37)=0, "", SUM(BH37,DI37,FJ37,HK37,JL37,LM37))</f>
-        <v/>
-      </c>
-      <c r="G37" s="6">
-        <f>IF(SUM(BG37,DH37,FI37,HJ37,JK37,LL37)=0, "", SUM(BG37,DH37,FI37,HJ37,JK37,LL37))</f>
-        <v/>
-      </c>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="6" t="n"/>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="43" t="n"/>
       <c r="J37" s="4" t="n"/>
@@ -47180,14 +46642,8 @@
         </is>
       </c>
       <c r="E38" s="6" t="n"/>
-      <c r="F38" s="8">
-        <f>IF(SUM(BH38,DI38,FJ38,HK38,JL38,LM38)=0, "", SUM(BH38,DI38,FJ38,HK38,JL38,LM38))</f>
-        <v/>
-      </c>
-      <c r="G38" s="6">
-        <f>IF(SUM(BG38,DH38,FI38,HJ38,JK38,LL38)=0, "", SUM(BG38,DH38,FI38,HJ38,JK38,LL38))</f>
-        <v/>
-      </c>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="6" t="n"/>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="43" t="n"/>
       <c r="J38" s="4" t="n"/>
@@ -47561,14 +47017,8 @@
         </is>
       </c>
       <c r="E39" s="6" t="n"/>
-      <c r="F39" s="8">
-        <f>IF(SUM(BH39,DI39,FJ39,HK39,JL39,LM39)=0, "", SUM(BH39,DI39,FJ39,HK39,JL39,LM39))</f>
-        <v/>
-      </c>
-      <c r="G39" s="6">
-        <f>IF(SUM(BG39,DH39,FI39,HJ39,JK39,LL39)=0, "", SUM(BG39,DH39,FI39,HJ39,JK39,LL39))</f>
-        <v/>
-      </c>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="6" t="n"/>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="43" t="n"/>
       <c r="J39" s="4" t="n"/>
@@ -47942,14 +47392,8 @@
         </is>
       </c>
       <c r="E40" s="6" t="n"/>
-      <c r="F40" s="8">
-        <f>IF(SUM(BH40,DI40,FJ40,HK40,JL40,LM40)=0, "", SUM(BH40,DI40,FJ40,HK40,JL40,LM40))</f>
-        <v/>
-      </c>
-      <c r="G40" s="6">
-        <f>IF(SUM(BG40,DH40,FI40,HJ40,JK40,LL40)=0, "", SUM(BG40,DH40,FI40,HJ40,JK40,LL40))</f>
-        <v/>
-      </c>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="6" t="n"/>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
       <c r="J40" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 05:56
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1311,13 +1311,13 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>7</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
@@ -6710,20 +6710,14 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I9" s="43" t="inlineStr">
-        <is>
-          <t>28.09</t>
-        </is>
-      </c>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="43" t="n"/>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="43" t="n"/>
       <c r="L9" s="4" t="n"/>
@@ -6742,9 +6736,7 @@
       <c r="Y9" s="43" t="n"/>
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
-      <c r="AB9" s="8" t="n">
-        <v>10</v>
-      </c>
+      <c r="AB9" s="8" t="n"/>
       <c r="AC9" s="43" t="n"/>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 06:01
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1310,14 +1310,12 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>8</v>
-      </c>
+      <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n">
         <v>7</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
@@ -6709,9 +6707,7 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>8</v>
-      </c>
+      <c r="E9" s="6" t="n"/>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="6" t="n">
         <v>1</v>
@@ -7015,14 +7011,8 @@
         <f>IF(COUNTA(IG9:JJ9)=0, "", COUNTA(IG9:JJ9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", IG9:JJ9))))</f>
         <v/>
       </c>
-      <c r="JM9" s="43" t="n">
-        <v>8</v>
-      </c>
-      <c r="JN9" s="43" t="inlineStr">
-        <is>
-          <t>28.09</t>
-        </is>
-      </c>
+      <c r="JM9" s="43" t="n"/>
+      <c r="JN9" s="43" t="n"/>
       <c r="JO9" s="43" t="n"/>
       <c r="JP9" s="43" t="n"/>
       <c r="JQ9" s="43" t="n"/>
@@ -7041,9 +7031,7 @@
       <c r="KD9" s="43" t="n"/>
       <c r="KE9" s="9" t="n"/>
       <c r="KF9" s="43" t="n"/>
-      <c r="KG9" s="44" t="n">
-        <v>8</v>
-      </c>
+      <c r="KG9" s="44" t="n"/>
       <c r="KH9" s="43" t="n"/>
       <c r="KI9" s="43" t="n"/>
       <c r="KJ9" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 06:02
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="24" t="n"/>
       <c r="L9" s="76" t="n"/>
@@ -35730,9 +35730,7 @@
       <c r="F9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="43" t="n"/>
       <c r="J9" s="4" t="n"/>
@@ -35754,11 +35752,7 @@
       <c r="Z9" s="43" t="n"/>
       <c r="AA9" s="9" t="n"/>
       <c r="AB9" s="8" t="n"/>
-      <c r="AC9" s="43" t="inlineStr">
-        <is>
-          <t>28.09m</t>
-        </is>
-      </c>
+      <c r="AC9" s="43" t="n"/>
       <c r="AD9" s="43" t="n"/>
       <c r="AE9" s="4" t="n"/>
       <c r="AF9" s="43" t="n"/>
@@ -47836,10 +47830,10 @@
         <v>1</v>
       </c>
       <c r="F9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="11" t="n">
         <v>2</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>3</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 06:03
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1321,9 +1321,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J9" s="4" t="n"/>
       <c r="K9" s="24" t="n"/>
       <c r="L9" s="76" t="n"/>
       <c r="M9" t="inlineStr">
@@ -6699,9 +6697,7 @@
       </c>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="8" t="n"/>
-      <c r="G9" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="43" t="n"/>
       <c r="J9" s="4" t="n"/>
@@ -6900,11 +6896,7 @@
       <c r="GC9" s="43" t="n"/>
       <c r="GD9" s="9" t="n"/>
       <c r="GE9" s="44" t="n"/>
-      <c r="GF9" s="43" t="inlineStr">
-        <is>
-          <t>28.09m</t>
-        </is>
-      </c>
+      <c r="GF9" s="43" t="n"/>
       <c r="GG9" s="43" t="n"/>
       <c r="GH9" s="43" t="n"/>
       <c r="GI9" s="43" t="n"/>
@@ -47821,12 +47813,8 @@
         </is>
       </c>
       <c r="E9" s="10" t="n"/>
-      <c r="F9" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="11" t="n"/>
       <c r="H9" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:38
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1321,7 +1321,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" s="24" t="n"/>
       <c r="L9" s="76" t="n"/>
       <c r="M9" t="inlineStr">
@@ -6696,7 +6698,9 @@
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="43" t="n"/>
@@ -7427,7 +7431,11 @@
       <c r="YL9" s="4" t="n"/>
       <c r="YM9" s="4" t="n"/>
       <c r="YN9" s="11" t="n"/>
-      <c r="YO9" s="4" t="n"/>
+      <c r="YO9" s="43" t="inlineStr">
+        <is>
+          <t>28.09</t>
+        </is>
+      </c>
       <c r="YP9" s="4" t="n"/>
       <c r="YQ9" s="4" t="n"/>
       <c r="YR9" s="4" t="n"/>
@@ -47812,9 +47820,13 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n"/>
+      <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F9" s="9" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="G9" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H9" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:39
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -6698,10 +6698,10 @@
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="43" t="n"/>
       <c r="J9" s="4" t="n"/>
@@ -7433,7 +7433,7 @@
       <c r="YN9" s="11" t="n"/>
       <c r="YO9" s="43" t="inlineStr">
         <is>
-          <t>28.09</t>
+          <t>28.09m</t>
         </is>
       </c>
       <c r="YP9" s="4" t="n"/>
@@ -47827,9 +47827,11 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="9" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" s="11" t="n">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:40
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1310,22 +1310,32 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n"/>
+      <c r="E9" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="G9" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H9" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K9" s="24" t="n"/>
-      <c r="L9" s="76" t="n"/>
+      <c r="K9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="76" t="inlineStr">
+        <is>
+          <t>Premiul I</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>2951</t>
@@ -6697,7 +6707,9 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
+      <c r="E9" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="6" t="n">
         <v>1</v>
@@ -6879,8 +6891,14 @@
         <f>IF(COUNTA(EE9:FH9)=0, "", COUNTA(EE9:FH9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE9:FH9))))</f>
         <v/>
       </c>
-      <c r="FK9" s="43" t="n"/>
-      <c r="FL9" s="43" t="n"/>
+      <c r="FK9" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="FL9" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM9" s="43" t="n"/>
       <c r="FN9" s="43" t="n"/>
       <c r="FO9" s="43" t="n"/>
@@ -6899,7 +6917,9 @@
       <c r="GB9" s="4" t="n"/>
       <c r="GC9" s="43" t="n"/>
       <c r="GD9" s="9" t="n"/>
-      <c r="GE9" s="44" t="n"/>
+      <c r="GE9" s="44" t="n">
+        <v>10</v>
+      </c>
       <c r="GF9" s="43" t="n"/>
       <c r="GG9" s="43" t="n"/>
       <c r="GH9" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:41
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="24" t="n">
         <v>1</v>
@@ -35747,7 +35747,9 @@
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
@@ -35954,7 +35956,11 @@
           <t>21.09m</t>
         </is>
       </c>
-      <c r="GG9" s="4" t="n"/>
+      <c r="GG9" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="GH9" s="4" t="n"/>
       <c r="GI9" s="4" t="n"/>
       <c r="GJ9" s="4" t="n"/>
@@ -47846,12 +47852,14 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n"/>
+      <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F9" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:42
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="24" t="n">
         <v>1</v>
@@ -35749,9 +35749,7 @@
         </is>
       </c>
       <c r="E9" s="6" t="n"/>
-      <c r="F9" s="8" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" s="8" t="n"/>
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
@@ -35958,11 +35956,7 @@
           <t>21.09m</t>
         </is>
       </c>
-      <c r="GG9" s="43" t="inlineStr">
-        <is>
-          <t>21.09</t>
-        </is>
-      </c>
+      <c r="GG9" s="43" t="n"/>
       <c r="GH9" s="4" t="n"/>
       <c r="GI9" s="4" t="n"/>
       <c r="GJ9" s="4" t="n"/>
@@ -47860,14 +47854,12 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="10" t="n">
-        <v>1</v>
-      </c>
+      <c r="E9" s="10" t="n"/>
       <c r="F9" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:43
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1310,32 +1310,22 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>10</v>
-      </c>
+      <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Promovat</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K9" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="76" t="inlineStr">
-        <is>
-          <t>Premiul I</t>
-        </is>
-      </c>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="76" t="n"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>2951</t>
@@ -6709,9 +6699,7 @@
           <t>126/76</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>10</v>
-      </c>
+      <c r="E9" s="6" t="n"/>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="6" t="n">
         <v>1</v>
@@ -6893,14 +6881,8 @@
         <f>IF(COUNTA(EE9:FH9)=0, "", COUNTA(EE9:FH9) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE9:FH9))))</f>
         <v/>
       </c>
-      <c r="FK9" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="FL9" s="43" t="inlineStr">
-        <is>
-          <t>18.09</t>
-        </is>
-      </c>
+      <c r="FK9" s="43" t="n"/>
+      <c r="FL9" s="43" t="n"/>
       <c r="FM9" s="43" t="n"/>
       <c r="FN9" s="43" t="n"/>
       <c r="FO9" s="43" t="n"/>
@@ -6919,9 +6901,7 @@
       <c r="GB9" s="4" t="n"/>
       <c r="GC9" s="43" t="n"/>
       <c r="GD9" s="9" t="n"/>
-      <c r="GE9" s="44" t="n">
-        <v>10</v>
-      </c>
+      <c r="GE9" s="44" t="n"/>
       <c r="GF9" s="43" t="n"/>
       <c r="GG9" s="43" t="n"/>
       <c r="GH9" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:44
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1349,20 +1349,30 @@
           <t>126/77</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n"/>
+      <c r="E10" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="G10" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J10" s="4" t="n"/>
-      <c r="K10" s="24" t="n"/>
-      <c r="L10" s="76" t="n"/>
+      <c r="K10" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="76" t="inlineStr">
+        <is>
+          <t>Premiul I</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t>6234</t>
@@ -7552,7 +7562,9 @@
           <t>126/77</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
+      <c r="E10" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F10" s="8" t="n"/>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="4" t="n"/>
@@ -7732,8 +7744,14 @@
         <f>IF(COUNTA(EE10:FH10)=0, "", COUNTA(EE10:FH10) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE10:FH10))))</f>
         <v/>
       </c>
-      <c r="FK10" s="43" t="n"/>
-      <c r="FL10" s="43" t="n"/>
+      <c r="FK10" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="FL10" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM10" s="43" t="n"/>
       <c r="FN10" s="43" t="n"/>
       <c r="FO10" s="43" t="n"/>
@@ -7752,7 +7770,9 @@
       <c r="GB10" s="4" t="n"/>
       <c r="GC10" s="43" t="n"/>
       <c r="GD10" s="9" t="n"/>
-      <c r="GE10" s="44" t="n"/>
+      <c r="GE10" s="44" t="n">
+        <v>10</v>
+      </c>
       <c r="GF10" s="43" t="n"/>
       <c r="GG10" s="43" t="n"/>
       <c r="GH10" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:45
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1435,20 +1435,30 @@
           <t>126/79</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n"/>
+      <c r="E12" s="4" t="n">
+        <v>9</v>
+      </c>
       <c r="F12" s="4" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="G12" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="H12" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J12" s="4" t="n"/>
-      <c r="K12" s="24" t="n"/>
-      <c r="L12" s="76" t="n"/>
+      <c r="K12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="76" t="inlineStr">
+        <is>
+          <t>Premiul II</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
           <t>9385</t>
@@ -9266,7 +9276,9 @@
           <t>126/79</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
+      <c r="E12" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="F12" s="8" t="n"/>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="4" t="n"/>
@@ -9446,8 +9458,14 @@
         <f>IF(COUNTA(EE12:FH12)=0, "", COUNTA(EE12:FH12) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE12:FH12))))</f>
         <v/>
       </c>
-      <c r="FK12" s="43" t="n"/>
-      <c r="FL12" s="43" t="n"/>
+      <c r="FK12" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="FL12" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM12" s="43" t="n"/>
       <c r="FN12" s="43" t="n"/>
       <c r="FO12" s="43" t="n"/>
@@ -9466,7 +9484,9 @@
       <c r="GB12" s="4" t="n"/>
       <c r="GC12" s="43" t="n"/>
       <c r="GD12" s="9" t="n"/>
-      <c r="GE12" s="44" t="n"/>
+      <c r="GE12" s="44" t="n">
+        <v>9</v>
+      </c>
       <c r="GF12" s="43" t="n"/>
       <c r="GG12" s="43" t="n"/>
       <c r="GH12" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:46
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1450,7 +1450,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" s="24" t="n">
         <v>2</v>
       </c>
@@ -9280,7 +9282,9 @@
         <v>9</v>
       </c>
       <c r="F12" s="8" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="G12" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="43" t="n"/>
       <c r="J12" s="4" t="n"/>
@@ -9841,7 +9845,11 @@
       <c r="SI12" s="4" t="n"/>
       <c r="SJ12" s="4" t="n"/>
       <c r="SK12" s="11" t="n"/>
-      <c r="SL12" s="4" t="n"/>
+      <c r="SL12" s="43" t="inlineStr">
+        <is>
+          <t>15.09m</t>
+        </is>
+      </c>
       <c r="SM12" s="4" t="n"/>
       <c r="SN12" s="4" t="n"/>
       <c r="SO12" s="4" t="n"/>
@@ -47967,8 +47975,12 @@
         </is>
       </c>
       <c r="E12" s="10" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="F12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H12" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:48
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1484,20 +1484,30 @@
           <t>126/80</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n"/>
+      <c r="E13" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="F13" s="4" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="G13" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="H13" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="24" t="n"/>
-      <c r="L13" s="76" t="n"/>
+      <c r="K13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="76" t="inlineStr">
+        <is>
+          <t>Premiul III</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t>2681</t>
@@ -10141,11 +10151,19 @@
           <t>126/80</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
+      <c r="E13" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="6" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="43" t="n"/>
+      <c r="H13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="43" t="n"/>
       <c r="L13" s="4" t="n"/>
@@ -10164,7 +10182,9 @@
       <c r="Y13" s="43" t="n"/>
       <c r="Z13" s="43" t="n"/>
       <c r="AA13" s="9" t="n"/>
-      <c r="AB13" s="8" t="n"/>
+      <c r="AB13" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="AC13" s="4" t="n"/>
       <c r="AD13" s="43" t="n"/>
       <c r="AE13" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:49
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="24" t="n">
         <v>3</v>
@@ -10158,7 +10158,7 @@
       </c>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>5</v>
@@ -10370,7 +10370,11 @@
       <c r="GC13" s="43" t="n"/>
       <c r="GD13" s="9" t="n"/>
       <c r="GE13" s="44" t="n"/>
-      <c r="GF13" s="43" t="n"/>
+      <c r="GF13" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="GG13" s="43" t="n"/>
       <c r="GH13" s="43" t="n"/>
       <c r="GI13" s="43" t="n"/>
@@ -48036,10 +48040,10 @@
       </c>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:50
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K13" s="24" t="n">
         <v>3</v>
@@ -10158,7 +10158,7 @@
       </c>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>5</v>
@@ -10913,7 +10913,11 @@
       <c r="YL13" s="4" t="n"/>
       <c r="YM13" s="4" t="n"/>
       <c r="YN13" s="11" t="n"/>
-      <c r="YO13" s="4" t="n"/>
+      <c r="YO13" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="YP13" s="4" t="n"/>
       <c r="YQ13" s="4" t="n"/>
       <c r="YR13" s="4" t="n"/>
@@ -48048,10 +48052,10 @@
       </c>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:51
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
         <v>3</v>
@@ -37338,7 +37338,9 @@
       </c>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="8" t="n"/>
-      <c r="G13" s="6" t="n"/>
+      <c r="G13" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="43" t="n"/>
       <c r="J13" s="4" t="n"/>
@@ -37537,7 +37539,11 @@
       <c r="GC13" s="4" t="n"/>
       <c r="GD13" s="4" t="n"/>
       <c r="GE13" s="11" t="n"/>
-      <c r="GF13" s="4" t="n"/>
+      <c r="GF13" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="GG13" s="4" t="n"/>
       <c r="GH13" s="4" t="n"/>
       <c r="GI13" s="4" t="n"/>
@@ -48056,10 +48062,10 @@
       </c>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H13" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:52
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1454,11 +1454,11 @@
         <v>1</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="76" t="inlineStr">
         <is>
-          <t>Premiul II</t>
+          <t>Premiul III</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1503,11 +1503,11 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
-          <t>Premiul III</t>
+          <t>Mențiune</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1533,20 +1533,30 @@
           <t>126/81</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="F14" s="4" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="G14" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="24" t="n"/>
-      <c r="L14" s="76" t="n"/>
+      <c r="K14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="76" t="inlineStr">
+        <is>
+          <t>Premiul I</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t>4658</t>
@@ -11036,7 +11046,9 @@
           <t>126/81</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
+      <c r="E14" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F14" s="8" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="4" t="n"/>
@@ -11216,8 +11228,14 @@
         <f>IF(COUNTA(EE14:FH14)=0, "", COUNTA(EE14:FH14) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE14:FH14))))</f>
         <v/>
       </c>
-      <c r="FK14" s="43" t="n"/>
-      <c r="FL14" s="43" t="n"/>
+      <c r="FK14" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="FL14" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM14" s="43" t="n"/>
       <c r="FN14" s="43" t="n"/>
       <c r="FO14" s="43" t="n"/>
@@ -11236,7 +11254,9 @@
       <c r="GB14" s="4" t="n"/>
       <c r="GC14" s="43" t="n"/>
       <c r="GD14" s="9" t="n"/>
-      <c r="GE14" s="44" t="n"/>
+      <c r="GE14" s="44" t="n">
+        <v>10</v>
+      </c>
       <c r="GF14" s="43" t="n"/>
       <c r="GG14" s="43" t="n"/>
       <c r="GH14" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:53
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1580,20 +1580,30 @@
           <t>126/82</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>8</v>
+      </c>
       <c r="F15" s="4" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="G15" s="6" t="n">
+        <v>8</v>
+      </c>
       <c r="H15" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J15" s="4" t="n"/>
-      <c r="K15" s="24" t="n"/>
-      <c r="L15" s="76" t="n"/>
+      <c r="K15" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="76" t="inlineStr">
+        <is>
+          <t>Mențiune</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>7891</t>
@@ -11903,7 +11913,9 @@
           <t>126/82</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
+      <c r="E15" s="6" t="n">
+        <v>8</v>
+      </c>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="4" t="n"/>
@@ -12083,8 +12095,14 @@
         <f>IF(COUNTA(EE15:FH15)=0, "", COUNTA(EE15:FH15) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE15:FH15))))</f>
         <v/>
       </c>
-      <c r="FK15" s="43" t="n"/>
-      <c r="FL15" s="43" t="n"/>
+      <c r="FK15" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="FL15" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM15" s="43" t="n"/>
       <c r="FN15" s="43" t="n"/>
       <c r="FO15" s="43" t="n"/>
@@ -12103,7 +12121,9 @@
       <c r="GB15" s="4" t="n"/>
       <c r="GC15" s="43" t="n"/>
       <c r="GD15" s="9" t="n"/>
-      <c r="GE15" s="44" t="n"/>
+      <c r="GE15" s="44" t="n">
+        <v>8</v>
+      </c>
       <c r="GF15" s="43" t="n"/>
       <c r="GG15" s="43" t="n"/>
       <c r="GH15" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:54
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1595,7 +1595,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K15" s="24" t="n">
         <v>4</v>
       </c>
@@ -11917,7 +11919,9 @@
         <v>8</v>
       </c>
       <c r="F15" s="8" t="n"/>
-      <c r="G15" s="6" t="n"/>
+      <c r="G15" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="43" t="n"/>
       <c r="J15" s="4" t="n"/>
@@ -12478,7 +12482,11 @@
       <c r="SI15" s="4" t="n"/>
       <c r="SJ15" s="4" t="n"/>
       <c r="SK15" s="11" t="n"/>
-      <c r="SL15" s="4" t="n"/>
+      <c r="SL15" s="43" t="inlineStr">
+        <is>
+          <t>15.09m</t>
+        </is>
+      </c>
       <c r="SM15" s="4" t="n"/>
       <c r="SN15" s="4" t="n"/>
       <c r="SO15" s="4" t="n"/>
@@ -48161,8 +48169,12 @@
         </is>
       </c>
       <c r="E15" s="10" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="F15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H15" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:55
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" s="24" t="n">
         <v>4</v>
@@ -38143,7 +38143,7 @@
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="43" t="n"/>
@@ -38284,7 +38284,11 @@
       <c r="EB15" s="9" t="n"/>
       <c r="EC15" s="10" t="n"/>
       <c r="ED15" s="11" t="n"/>
-      <c r="EE15" s="4" t="n"/>
+      <c r="EE15" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="EF15" s="4" t="n"/>
       <c r="EG15" s="4" t="n"/>
       <c r="EH15" s="4" t="n"/>
@@ -48180,10 +48184,10 @@
       </c>
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:56
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1640,7 +1640,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" s="24" t="n"/>
       <c r="L16" s="76" t="n"/>
       <c r="M16" t="inlineStr">
@@ -12780,7 +12782,9 @@
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="8" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="G16" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -12802,7 +12806,11 @@
       <c r="Z16" s="43" t="n"/>
       <c r="AA16" s="9" t="n"/>
       <c r="AB16" s="8" t="n"/>
-      <c r="AC16" s="4" t="n"/>
+      <c r="AC16" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="AD16" s="43" t="n"/>
       <c r="AE16" s="4" t="n"/>
       <c r="AF16" s="43" t="n"/>
@@ -48215,8 +48223,12 @@
         </is>
       </c>
       <c r="E16" s="10" t="n"/>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="F16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H16" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:57
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K16" s="24" t="n"/>
       <c r="L16" s="76" t="n"/>
@@ -12783,7 +12783,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
@@ -13231,7 +13231,11 @@
       <c r="OG16" s="4" t="n"/>
       <c r="OH16" s="4" t="n"/>
       <c r="OI16" s="11" t="n"/>
-      <c r="OJ16" s="4" t="n"/>
+      <c r="OJ16" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="OK16" s="4" t="n"/>
       <c r="OL16" s="4" t="n"/>
       <c r="OM16" s="4" t="n"/>
@@ -48232,10 +48236,10 @@
       </c>
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:58
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K16" s="24" t="n"/>
       <c r="L16" s="76" t="n"/>
@@ -38559,7 +38559,9 @@
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="8" t="n"/>
-      <c r="G16" s="6" t="n"/>
+      <c r="G16" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -38758,7 +38760,11 @@
       <c r="GC16" s="4" t="n"/>
       <c r="GD16" s="4" t="n"/>
       <c r="GE16" s="11" t="n"/>
-      <c r="GF16" s="4" t="n"/>
+      <c r="GF16" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="GG16" s="4" t="n"/>
       <c r="GH16" s="4" t="n"/>
       <c r="GI16" s="4" t="n"/>
@@ -48244,10 +48250,10 @@
       </c>
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H16" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 11:59
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1668,20 +1668,30 @@
           <t>126/84</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n"/>
+      <c r="E17" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="F17" s="4" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="G17" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="H17" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="24" t="n"/>
-      <c r="L17" s="76" t="n"/>
+      <c r="K17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="76" t="inlineStr">
+        <is>
+          <t>Mențiune</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t>9042</t>
@@ -13653,11 +13663,19 @@
           <t>126/84</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
+      <c r="E17" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="6" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="43" t="n"/>
+      <c r="H17" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" s="43" t="inlineStr">
+        <is>
+          <t>25.09</t>
+        </is>
+      </c>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="43" t="n"/>
       <c r="L17" s="4" t="n"/>
@@ -13676,7 +13694,9 @@
       <c r="Y17" s="43" t="n"/>
       <c r="Z17" s="43" t="n"/>
       <c r="AA17" s="9" t="n"/>
-      <c r="AB17" s="8" t="n"/>
+      <c r="AB17" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="AC17" s="4" t="n"/>
       <c r="AD17" s="43" t="n"/>
       <c r="AE17" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:01
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K16" s="24" t="n"/>
       <c r="L16" s="76" t="n"/>
@@ -12793,7 +12793,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="43" t="n"/>
@@ -13010,11 +13010,7 @@
           <t>25.09m</t>
         </is>
       </c>
-      <c r="GG16" s="43" t="inlineStr">
-        <is>
-          <t>25.09m</t>
-        </is>
-      </c>
+      <c r="GG16" s="43" t="n"/>
       <c r="GH16" s="43" t="n"/>
       <c r="GI16" s="43" t="n"/>
       <c r="GJ16" s="43" t="n"/>
@@ -48278,10 +48274,10 @@
       </c>
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H16" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:02
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1683,7 +1683,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="24" t="n">
         <v>5</v>
       </c>
@@ -13667,7 +13669,9 @@
         <v>5</v>
       </c>
       <c r="F17" s="8" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="G17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" s="4" t="n">
         <v>5</v>
       </c>
@@ -13697,7 +13701,11 @@
       <c r="AB17" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="AC17" s="4" t="n"/>
+      <c r="AC17" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="AD17" s="43" t="n"/>
       <c r="AE17" s="4" t="n"/>
       <c r="AF17" s="43" t="n"/>
@@ -48301,8 +48309,12 @@
         </is>
       </c>
       <c r="E17" s="10" t="n"/>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="F17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:03
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K17" s="24" t="n">
         <v>5</v>
@@ -13670,7 +13670,7 @@
       </c>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17" s="4" t="n">
         <v>5</v>
@@ -14126,7 +14126,11 @@
       <c r="OG17" s="4" t="n"/>
       <c r="OH17" s="4" t="n"/>
       <c r="OI17" s="11" t="n"/>
-      <c r="OJ17" s="4" t="n"/>
+      <c r="OJ17" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="OK17" s="4" t="n"/>
       <c r="OL17" s="4" t="n"/>
       <c r="OM17" s="4" t="n"/>
@@ -48318,10 +48322,10 @@
       </c>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:04
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K17" s="24" t="n">
         <v>5</v>
@@ -13670,7 +13670,7 @@
       </c>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" s="4" t="n">
         <v>5</v>
@@ -14252,7 +14252,11 @@
       <c r="SI17" s="4" t="n"/>
       <c r="SJ17" s="4" t="n"/>
       <c r="SK17" s="11" t="n"/>
-      <c r="SL17" s="4" t="n"/>
+      <c r="SL17" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="SM17" s="4" t="n"/>
       <c r="SN17" s="4" t="n"/>
       <c r="SO17" s="4" t="n"/>
@@ -48326,10 +48330,10 @@
       </c>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:05
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K17" s="24" t="n">
         <v>5</v>
@@ -38996,7 +38996,9 @@
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="8" t="n"/>
-      <c r="G17" s="6" t="n"/>
+      <c r="G17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="43" t="n"/>
       <c r="J17" s="4" t="n"/>
@@ -39195,7 +39197,11 @@
       <c r="GC17" s="4" t="n"/>
       <c r="GD17" s="4" t="n"/>
       <c r="GE17" s="11" t="n"/>
-      <c r="GF17" s="4" t="n"/>
+      <c r="GF17" s="43" t="inlineStr">
+        <is>
+          <t>24.09m</t>
+        </is>
+      </c>
       <c r="GG17" s="4" t="n"/>
       <c r="GH17" s="4" t="n"/>
       <c r="GI17" s="4" t="n"/>
@@ -48338,10 +48344,10 @@
       </c>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:06
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K17" s="24" t="n">
         <v>5</v>
@@ -38997,7 +38997,7 @@
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="43" t="n"/>
@@ -39138,7 +39138,11 @@
       <c r="EB17" s="9" t="n"/>
       <c r="EC17" s="10" t="n"/>
       <c r="ED17" s="11" t="n"/>
-      <c r="EE17" s="4" t="n"/>
+      <c r="EE17" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="EF17" s="4" t="n"/>
       <c r="EG17" s="4" t="n"/>
       <c r="EH17" s="4" t="n"/>
@@ -48344,10 +48348,10 @@
       </c>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H17" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:07
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1728,7 +1728,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="24" t="n"/>
       <c r="L18" s="76" t="n"/>
       <c r="M18" t="inlineStr">
@@ -14558,7 +14560,9 @@
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="8" t="n"/>
-      <c r="G18" s="6" t="n"/>
+      <c r="G18" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="43" t="n"/>
       <c r="J18" s="4" t="n"/>
@@ -14580,7 +14584,11 @@
       <c r="Z18" s="43" t="n"/>
       <c r="AA18" s="9" t="n"/>
       <c r="AB18" s="8" t="n"/>
-      <c r="AC18" s="4" t="n"/>
+      <c r="AC18" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="AD18" s="43" t="n"/>
       <c r="AE18" s="4" t="n"/>
       <c r="AF18" s="43" t="n"/>
@@ -48383,8 +48391,12 @@
         </is>
       </c>
       <c r="E18" s="10" t="n"/>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="F18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H18" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:08
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K18" s="24" t="n"/>
       <c r="L18" s="76" t="n"/>
@@ -39401,7 +39401,9 @@
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="8" t="n"/>
-      <c r="G18" s="6" t="n"/>
+      <c r="G18" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="43" t="n"/>
       <c r="J18" s="4" t="n"/>
@@ -39600,7 +39602,11 @@
       <c r="GC18" s="4" t="n"/>
       <c r="GD18" s="4" t="n"/>
       <c r="GE18" s="11" t="n"/>
-      <c r="GF18" s="4" t="n"/>
+      <c r="GF18" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="GG18" s="4" t="n"/>
       <c r="GH18" s="4" t="n"/>
       <c r="GI18" s="4" t="n"/>
@@ -48400,10 +48406,10 @@
       </c>
       <c r="E18" s="10" t="n"/>
       <c r="F18" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H18" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:10
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1771,7 +1771,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" s="24" t="n">
         <v>3</v>
       </c>
@@ -15433,7 +15435,9 @@
         <v>9</v>
       </c>
       <c r="F19" s="8" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="G19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="43" t="n"/>
       <c r="J19" s="4" t="n"/>
@@ -15994,7 +15998,11 @@
       <c r="SI19" s="4" t="n"/>
       <c r="SJ19" s="4" t="n"/>
       <c r="SK19" s="11" t="n"/>
-      <c r="SL19" s="4" t="n"/>
+      <c r="SL19" s="43" t="inlineStr">
+        <is>
+          <t>15.09m</t>
+        </is>
+      </c>
       <c r="SM19" s="4" t="n"/>
       <c r="SN19" s="4" t="n"/>
       <c r="SO19" s="4" t="n"/>
@@ -48457,8 +48465,12 @@
         </is>
       </c>
       <c r="E19" s="10" t="n"/>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="F19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H19" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:11
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K19" s="24" t="n">
         <v>3</v>
@@ -39810,7 +39810,7 @@
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>1</v>
@@ -39954,7 +39954,11 @@
       <c r="EB19" s="9" t="n"/>
       <c r="EC19" s="10" t="n"/>
       <c r="ED19" s="11" t="n"/>
-      <c r="EE19" s="4" t="n"/>
+      <c r="EE19" s="43" t="inlineStr">
+        <is>
+          <t>22.09</t>
+        </is>
+      </c>
       <c r="EF19" s="4" t="n"/>
       <c r="EG19" s="4" t="n"/>
       <c r="EH19" s="4" t="n"/>
@@ -48477,13 +48481,13 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:12
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1820,7 +1820,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="24" t="n">
         <v>3</v>
       </c>
@@ -40220,7 +40222,9 @@
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="8" t="n"/>
+      <c r="F20" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G20" s="6" t="n"/>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="43" t="n"/>
@@ -40420,7 +40424,11 @@
       <c r="GC20" s="4" t="n"/>
       <c r="GD20" s="4" t="n"/>
       <c r="GE20" s="11" t="n"/>
-      <c r="GF20" s="4" t="n"/>
+      <c r="GF20" s="43" t="inlineStr">
+        <is>
+          <t>23.09</t>
+        </is>
+      </c>
       <c r="GG20" s="4" t="n"/>
       <c r="GH20" s="4" t="n"/>
       <c r="GI20" s="4" t="n"/>
@@ -48534,9 +48542,13 @@
           <t>126/87</t>
         </is>
       </c>
-      <c r="E20" s="10" t="n"/>
+      <c r="E20" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F20" s="9" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H20" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:13
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -39832,10 +39832,10 @@
       </c>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>1</v>
       </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="43" t="n"/>
@@ -39978,7 +39978,7 @@
       <c r="ED19" s="11" t="n"/>
       <c r="EE19" s="43" t="inlineStr">
         <is>
-          <t>22.09</t>
+          <t>22.09m</t>
         </is>
       </c>
       <c r="EF19" s="4" t="n"/>
@@ -48509,10 +48509,10 @@
         </is>
       </c>
       <c r="E19" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" s="11" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:14
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1854,20 +1854,30 @@
           <t>126/88</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n"/>
+      <c r="E21" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="F21" s="4" t="n"/>
-      <c r="G21" s="6" t="n"/>
+      <c r="G21" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="H21" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J21" s="4" t="n"/>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="76" t="n"/>
+      <c r="K21" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L21" s="76" t="inlineStr">
+        <is>
+          <t>Mențiune</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>2322</t>
@@ -17163,11 +17173,19 @@
           <t>126/88</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
+      <c r="E21" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="6" t="n"/>
-      <c r="H21" s="4" t="n"/>
-      <c r="I21" s="43" t="n"/>
+      <c r="H21" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="43" t="n"/>
       <c r="L21" s="4" t="n"/>
@@ -17186,7 +17204,9 @@
       <c r="Y21" s="43" t="n"/>
       <c r="Z21" s="43" t="n"/>
       <c r="AA21" s="9" t="n"/>
-      <c r="AB21" s="8" t="n"/>
+      <c r="AB21" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="AC21" s="4" t="n"/>
       <c r="AD21" s="43" t="n"/>
       <c r="AE21" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:15
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="24" t="n">
         <v>7</v>
@@ -17180,7 +17180,7 @@
       </c>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>5</v>
@@ -17392,7 +17392,11 @@
       <c r="GC21" s="43" t="n"/>
       <c r="GD21" s="9" t="n"/>
       <c r="GE21" s="44" t="n"/>
-      <c r="GF21" s="43" t="n"/>
+      <c r="GF21" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="GG21" s="43" t="n"/>
       <c r="GH21" s="43" t="n"/>
       <c r="GI21" s="43" t="n"/>
@@ -48604,10 +48608,10 @@
       </c>
       <c r="E21" s="10" t="n"/>
       <c r="F21" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:17
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K21" s="24" t="n">
         <v>7</v>
@@ -17178,7 +17178,9 @@
       <c r="E21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G21" s="6" t="n">
         <v>4</v>
       </c>
@@ -17758,7 +17760,11 @@
       <c r="SI21" s="4" t="n"/>
       <c r="SJ21" s="4" t="n"/>
       <c r="SK21" s="11" t="n"/>
-      <c r="SL21" s="4" t="n"/>
+      <c r="SL21" s="43" t="inlineStr">
+        <is>
+          <t>22.09</t>
+        </is>
+      </c>
       <c r="SM21" s="4" t="n"/>
       <c r="SN21" s="4" t="n"/>
       <c r="SO21" s="4" t="n"/>
@@ -48614,12 +48620,14 @@
           <t>126/88</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n"/>
+      <c r="E21" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" s="9" t="n">
         <v>4</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H21" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:18
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
         <v>7</v>
@@ -17179,7 +17179,7 @@
         <v>5</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>4</v>
@@ -17882,7 +17882,11 @@
       <c r="WK21" s="4" t="n"/>
       <c r="WL21" s="4" t="n"/>
       <c r="WM21" s="11" t="n"/>
-      <c r="WN21" s="4" t="n"/>
+      <c r="WN21" s="43" t="inlineStr">
+        <is>
+          <t>25.09</t>
+        </is>
+      </c>
       <c r="WO21" s="4" t="n"/>
       <c r="WP21" s="4" t="n"/>
       <c r="WQ21" s="4" t="n"/>
@@ -48621,13 +48625,13 @@
         </is>
       </c>
       <c r="E21" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>4</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H21" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:20
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1914,7 +1914,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J22" s="4" t="n"/>
+      <c r="J22" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" s="24" t="n"/>
       <c r="L22" s="76" t="n"/>
       <c r="M22" t="inlineStr">
@@ -18061,7 +18063,9 @@
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="43" t="n"/>
@@ -18497,7 +18501,11 @@
       <c r="OG22" s="4" t="n"/>
       <c r="OH22" s="4" t="n"/>
       <c r="OI22" s="11" t="n"/>
-      <c r="OJ22" s="4" t="n"/>
+      <c r="OJ22" s="43" t="inlineStr">
+        <is>
+          <t>22.09</t>
+        </is>
+      </c>
       <c r="OK22" s="4" t="n"/>
       <c r="OL22" s="4" t="n"/>
       <c r="OM22" s="4" t="n"/>
@@ -48658,9 +48666,13 @@
           <t>126/89</t>
         </is>
       </c>
-      <c r="E22" s="10" t="n"/>
+      <c r="E22" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F22" s="9" t="n"/>
-      <c r="G22" s="11" t="n"/>
+      <c r="G22" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H22" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:21
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -18063,10 +18063,10 @@
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="6" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="43" t="n"/>
       <c r="J22" s="4" t="n"/>
@@ -18503,7 +18503,7 @@
       <c r="OI22" s="11" t="n"/>
       <c r="OJ22" s="43" t="inlineStr">
         <is>
-          <t>22.09</t>
+          <t>22.09m</t>
         </is>
       </c>
       <c r="OK22" s="4" t="n"/>
@@ -48666,10 +48666,10 @@
           <t>126/89</t>
         </is>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="9" t="n"/>
       <c r="G22" s="11" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:22
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="24" t="n"/>
       <c r="L22" s="76" t="n"/>
@@ -41040,7 +41040,9 @@
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
-      <c r="F22" s="8" t="n"/>
+      <c r="F22" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="43" t="n"/>
@@ -41240,7 +41242,11 @@
       <c r="GC22" s="4" t="n"/>
       <c r="GD22" s="4" t="n"/>
       <c r="GE22" s="11" t="n"/>
-      <c r="GF22" s="4" t="n"/>
+      <c r="GF22" s="43" t="inlineStr">
+        <is>
+          <t>23.09</t>
+        </is>
+      </c>
       <c r="GG22" s="4" t="n"/>
       <c r="GH22" s="4" t="n"/>
       <c r="GI22" s="4" t="n"/>
@@ -48670,12 +48676,14 @@
           <t>126/89</t>
         </is>
       </c>
-      <c r="E22" s="10" t="n"/>
+      <c r="E22" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="F22" s="9" t="n">
         <v>2</v>
       </c>
       <c r="G22" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:23
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,11 +1503,11 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
-          <t>Mențiune</t>
+          <t>Membru</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1687,11 +1687,11 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
-          <t>Mențiune</t>
+          <t>Membru</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1873,11 +1873,11 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
-          <t>Mențiune</t>
+          <t>Membru</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1942,20 +1942,30 @@
           <t>126/90</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n"/>
+      <c r="E23" s="4" t="n">
+        <v>7</v>
+      </c>
       <c r="F23" s="4" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="G23" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="H23" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J23" s="4" t="n"/>
-      <c r="K23" s="24" t="n"/>
-      <c r="L23" s="76" t="n"/>
+      <c r="K23" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L23" s="76" t="inlineStr">
+        <is>
+          <t>Mențiune</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>5706</t>
@@ -18923,7 +18933,9 @@
           <t>126/90</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
+      <c r="E23" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="4" t="n"/>
@@ -19103,8 +19115,14 @@
         <f>IF(COUNTA(EE23:FH23)=0, "", COUNTA(EE23:FH23) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE23:FH23))))</f>
         <v/>
       </c>
-      <c r="FK23" s="43" t="n"/>
-      <c r="FL23" s="43" t="n"/>
+      <c r="FK23" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="FL23" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM23" s="43" t="n"/>
       <c r="FN23" s="43" t="n"/>
       <c r="FO23" s="43" t="n"/>
@@ -19123,7 +19141,9 @@
       <c r="GB23" s="4" t="n"/>
       <c r="GC23" s="43" t="n"/>
       <c r="GD23" s="9" t="n"/>
-      <c r="GE23" s="44" t="n"/>
+      <c r="GE23" s="44" t="n">
+        <v>7</v>
+      </c>
       <c r="GF23" s="43" t="n"/>
       <c r="GG23" s="43" t="n"/>
       <c r="GH23" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:24
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1957,7 +1957,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" s="24" t="n">
         <v>7</v>
       </c>
@@ -18937,7 +18939,9 @@
         <v>7</v>
       </c>
       <c r="F23" s="8" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="G23" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
       <c r="J23" s="4" t="n"/>
@@ -19380,7 +19384,11 @@
       <c r="OG23" s="4" t="n"/>
       <c r="OH23" s="4" t="n"/>
       <c r="OI23" s="11" t="n"/>
-      <c r="OJ23" s="4" t="n"/>
+      <c r="OJ23" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="OK23" s="4" t="n"/>
       <c r="OL23" s="4" t="n"/>
       <c r="OM23" s="4" t="n"/>
@@ -48741,8 +48749,12 @@
         </is>
       </c>
       <c r="E23" s="10" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="F23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:25
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" s="24" t="n">
         <v>7</v>
@@ -18940,7 +18940,7 @@
       </c>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
@@ -19687,7 +19687,11 @@
       <c r="YL23" s="4" t="n"/>
       <c r="YM23" s="4" t="n"/>
       <c r="YN23" s="11" t="n"/>
-      <c r="YO23" s="4" t="n"/>
+      <c r="YO23" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="YP23" s="4" t="n"/>
       <c r="YQ23" s="4" t="n"/>
       <c r="YR23" s="4" t="n"/>
@@ -48754,10 +48758,10 @@
       </c>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:26
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K23" s="24" t="n">
         <v>7</v>
@@ -41472,7 +41472,9 @@
       </c>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="8" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="G23" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
       <c r="J23" s="4" t="n"/>
@@ -41671,7 +41673,11 @@
       <c r="GC23" s="4" t="n"/>
       <c r="GD23" s="4" t="n"/>
       <c r="GE23" s="11" t="n"/>
-      <c r="GF23" s="4" t="n"/>
+      <c r="GF23" s="43" t="inlineStr">
+        <is>
+          <t>21.09m</t>
+        </is>
+      </c>
       <c r="GG23" s="4" t="n"/>
       <c r="GH23" s="4" t="n"/>
       <c r="GI23" s="4" t="n"/>
@@ -48762,10 +48768,10 @@
       </c>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H23" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:27
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K23" s="24" t="n">
         <v>7</v>
@@ -41473,7 +41473,7 @@
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="43" t="n"/>
@@ -41619,7 +41619,11 @@
           <t>22.09m</t>
         </is>
       </c>
-      <c r="EF23" s="4" t="n"/>
+      <c r="EF23" s="43" t="inlineStr">
+        <is>
+          <t>24.09m</t>
+        </is>
+      </c>
       <c r="EG23" s="4" t="n"/>
       <c r="EH23" s="4" t="n"/>
       <c r="EI23" s="4" t="n"/>
@@ -48772,10 +48776,10 @@
       </c>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H23" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:29
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2002,7 +2002,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" s="24" t="n"/>
       <c r="L24" s="76" t="n"/>
       <c r="M24" t="inlineStr">
@@ -19812,7 +19814,9 @@
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="8" t="n"/>
-      <c r="G24" s="6" t="n"/>
+      <c r="G24" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="43" t="n"/>
       <c r="J24" s="4" t="n"/>
@@ -20365,7 +20369,11 @@
       <c r="SI24" s="4" t="n"/>
       <c r="SJ24" s="4" t="n"/>
       <c r="SK24" s="11" t="n"/>
-      <c r="SL24" s="4" t="n"/>
+      <c r="SL24" s="43" t="inlineStr">
+        <is>
+          <t>15.09m</t>
+        </is>
+      </c>
       <c r="SM24" s="4" t="n"/>
       <c r="SN24" s="4" t="n"/>
       <c r="SO24" s="4" t="n"/>
@@ -48807,8 +48815,12 @@
         </is>
       </c>
       <c r="E24" s="10" t="n"/>
-      <c r="F24" s="9" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="F24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H24" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:30
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -2030,20 +2030,30 @@
           <t>126/92</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n"/>
+      <c r="E25" s="4" t="n">
+        <v>7</v>
+      </c>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="6" t="n"/>
+      <c r="G25" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="H25" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J25" s="4" t="n"/>
-      <c r="K25" s="24" t="n"/>
-      <c r="L25" s="76" t="n"/>
+      <c r="K25" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L25" s="76" t="inlineStr">
+        <is>
+          <t>Mențiune</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>8367</t>
@@ -20665,11 +20675,19 @@
           <t>126/92</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
+      <c r="E25" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="6" t="n"/>
-      <c r="H25" s="4" t="n"/>
-      <c r="I25" s="43" t="n"/>
+      <c r="H25" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I25" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="43" t="n"/>
       <c r="L25" s="4" t="n"/>
@@ -20688,7 +20706,9 @@
       <c r="Y25" s="43" t="n"/>
       <c r="Z25" s="43" t="n"/>
       <c r="AA25" s="9" t="n"/>
-      <c r="AB25" s="8" t="n"/>
+      <c r="AB25" s="8" t="n">
+        <v>7</v>
+      </c>
       <c r="AC25" s="4" t="n"/>
       <c r="AD25" s="43" t="n"/>
       <c r="AE25" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:31
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1961,11 +1961,11 @@
         <v>7</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L23" s="76" t="inlineStr">
         <is>
-          <t>Mențiune</t>
+          <t>Membru</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2031,11 +2031,11 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="6" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="H25" s="4" t="n">
         <v>10</v>
@@ -20676,7 +20676,7 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="6" t="n"/>
@@ -20865,8 +20865,14 @@
         <f>IF(COUNTA(EE25:FH25)=0, "", COUNTA(EE25:FH25) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE25:FH25))))</f>
         <v/>
       </c>
-      <c r="FK25" s="43" t="n"/>
-      <c r="FL25" s="43" t="n"/>
+      <c r="FK25" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="FL25" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM25" s="43" t="n"/>
       <c r="FN25" s="43" t="n"/>
       <c r="FO25" s="43" t="n"/>
@@ -20885,7 +20891,9 @@
       <c r="GB25" s="4" t="n"/>
       <c r="GC25" s="43" t="n"/>
       <c r="GD25" s="9" t="n"/>
-      <c r="GE25" s="44" t="n"/>
+      <c r="GE25" s="44" t="n">
+        <v>8</v>
+      </c>
       <c r="GF25" s="43" t="n"/>
       <c r="GG25" s="43" t="n"/>
       <c r="GH25" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:32
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2088,7 +2088,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" s="24" t="n"/>
       <c r="L26" s="76" t="n"/>
       <c r="M26" t="inlineStr">
@@ -21542,7 +21544,9 @@
       </c>
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="8" t="n"/>
-      <c r="G26" s="6" t="n"/>
+      <c r="G26" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="43" t="n"/>
       <c r="J26" s="4" t="n"/>
@@ -21564,7 +21568,11 @@
       <c r="Z26" s="43" t="n"/>
       <c r="AA26" s="9" t="n"/>
       <c r="AB26" s="8" t="n"/>
-      <c r="AC26" s="4" t="n"/>
+      <c r="AC26" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="AD26" s="43" t="n"/>
       <c r="AE26" s="4" t="n"/>
       <c r="AF26" s="43" t="n"/>
@@ -48909,8 +48917,12 @@
         </is>
       </c>
       <c r="E26" s="10" t="n"/>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="F26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H26" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:33
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K26" s="24" t="n"/>
       <c r="L26" s="76" t="n"/>
@@ -21545,7 +21545,7 @@
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="43" t="n"/>
@@ -22048,7 +22048,11 @@
       <c r="QH26" s="4" t="n"/>
       <c r="QI26" s="4" t="n"/>
       <c r="QJ26" s="11" t="n"/>
-      <c r="QK26" s="4" t="n"/>
+      <c r="QK26" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="QL26" s="4" t="n"/>
       <c r="QM26" s="4" t="n"/>
       <c r="QN26" s="4" t="n"/>
@@ -48922,10 +48926,10 @@
       </c>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:34
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K26" s="24" t="n"/>
       <c r="L26" s="76" t="n"/>
@@ -21545,7 +21545,7 @@
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="43" t="n"/>
@@ -22233,7 +22233,11 @@
       <c r="WK26" s="4" t="n"/>
       <c r="WL26" s="4" t="n"/>
       <c r="WM26" s="11" t="n"/>
-      <c r="WN26" s="4" t="n"/>
+      <c r="WN26" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="WO26" s="4" t="n"/>
       <c r="WP26" s="4" t="n"/>
       <c r="WQ26" s="4" t="n"/>
@@ -48930,10 +48934,10 @@
       </c>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H26" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:35
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -2116,20 +2116,30 @@
           <t>126/94</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n"/>
+      <c r="E27" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="F27" s="4" t="n"/>
-      <c r="G27" s="6" t="n"/>
+      <c r="G27" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="H27" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J27" s="4" t="n"/>
-      <c r="K27" s="24" t="n"/>
-      <c r="L27" s="76" t="n"/>
+      <c r="K27" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="L27" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>9032</t>
@@ -22411,11 +22421,19 @@
           <t>126/94</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
+      <c r="E27" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="6" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="43" t="n"/>
+      <c r="H27" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I27" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="43" t="n"/>
       <c r="L27" s="4" t="n"/>
@@ -22434,7 +22452,9 @@
       <c r="Y27" s="43" t="n"/>
       <c r="Z27" s="43" t="n"/>
       <c r="AA27" s="9" t="n"/>
-      <c r="AB27" s="8" t="n"/>
+      <c r="AB27" s="8" t="n">
+        <v>6</v>
+      </c>
       <c r="AC27" s="4" t="n"/>
       <c r="AD27" s="43" t="n"/>
       <c r="AE27" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:36
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2178,7 +2178,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J28" s="4" t="n"/>
+      <c r="J28" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" s="24" t="n">
         <v>3</v>
       </c>
@@ -43473,7 +43475,9 @@
       </c>
       <c r="E28" s="6" t="n"/>
       <c r="F28" s="8" t="n"/>
-      <c r="G28" s="6" t="n"/>
+      <c r="G28" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="43" t="n"/>
       <c r="J28" s="4" t="n"/>
@@ -43613,7 +43617,11 @@
       <c r="EB28" s="9" t="n"/>
       <c r="EC28" s="10" t="n"/>
       <c r="ED28" s="11" t="n"/>
-      <c r="EE28" s="4" t="n"/>
+      <c r="EE28" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="EF28" s="4" t="n"/>
       <c r="EG28" s="4" t="n"/>
       <c r="EH28" s="4" t="n"/>
@@ -49039,8 +49047,12 @@
         </is>
       </c>
       <c r="E28" s="10" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="11" t="n"/>
+      <c r="F28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H28" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:37
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -2212,20 +2212,30 @@
           <t>126/96</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n"/>
+      <c r="E29" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="F29" s="4" t="n"/>
-      <c r="G29" s="6" t="n"/>
+      <c r="G29" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="H29" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J29" s="4" t="n"/>
-      <c r="K29" s="24" t="n"/>
-      <c r="L29" s="76" t="n"/>
+      <c r="K29" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="L29" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>4444</t>
@@ -24147,11 +24157,19 @@
           <t>126/96</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
+      <c r="E29" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="6" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="43" t="n"/>
+      <c r="H29" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I29" s="43" t="inlineStr">
+        <is>
+          <t>21.09</t>
+        </is>
+      </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="43" t="n"/>
       <c r="L29" s="4" t="n"/>
@@ -24170,7 +24188,9 @@
       <c r="Y29" s="43" t="n"/>
       <c r="Z29" s="43" t="n"/>
       <c r="AA29" s="9" t="n"/>
-      <c r="AB29" s="8" t="n"/>
+      <c r="AB29" s="8" t="n">
+        <v>6</v>
+      </c>
       <c r="AC29" s="4" t="n"/>
       <c r="AD29" s="43" t="n"/>
       <c r="AE29" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:38
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2259,20 +2259,30 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
+      <c r="E30" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="F30" s="4" t="n"/>
-      <c r="G30" s="6" t="n"/>
+      <c r="G30" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="H30" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Corigent / Repetent</t>
         </is>
       </c>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="24" t="n"/>
-      <c r="L30" s="76" t="n"/>
+      <c r="K30" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="L30" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>7508</t>
@@ -25014,7 +25024,9 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
+      <c r="E30" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n"/>
@@ -25194,8 +25206,14 @@
         <f>IF(COUNTA(EE30:FH30)=0, "", COUNTA(EE30:FH30) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE30:FH30))))</f>
         <v/>
       </c>
-      <c r="FK30" s="43" t="n"/>
-      <c r="FL30" s="43" t="n"/>
+      <c r="FK30" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="FL30" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM30" s="43" t="n"/>
       <c r="FN30" s="43" t="n"/>
       <c r="FO30" s="43" t="n"/>
@@ -25214,7 +25232,9 @@
       <c r="GB30" s="4" t="n"/>
       <c r="GC30" s="43" t="n"/>
       <c r="GD30" s="9" t="n"/>
-      <c r="GE30" s="44" t="n"/>
+      <c r="GE30" s="44" t="n">
+        <v>4</v>
+      </c>
       <c r="GF30" s="43" t="n"/>
       <c r="GG30" s="43" t="n"/>
       <c r="GH30" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:39
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2364,7 +2364,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J32" s="4" t="n"/>
+      <c r="J32" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" s="24" t="n"/>
       <c r="L32" s="76" t="n"/>
       <c r="M32" t="inlineStr">
@@ -26750,7 +26752,9 @@
       </c>
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="8" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="G32" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="43" t="n"/>
       <c r="J32" s="4" t="n"/>
@@ -27480,7 +27484,11 @@
       <c r="YL32" s="4" t="n"/>
       <c r="YM32" s="4" t="n"/>
       <c r="YN32" s="11" t="n"/>
-      <c r="YO32" s="4" t="n"/>
+      <c r="YO32" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="YP32" s="4" t="n"/>
       <c r="YQ32" s="4" t="n"/>
       <c r="YR32" s="4" t="n"/>
@@ -49223,8 +49231,12 @@
         </is>
       </c>
       <c r="E32" s="10" t="n"/>
-      <c r="F32" s="9" t="n"/>
-      <c r="G32" s="11" t="n"/>
+      <c r="F32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H32" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:40
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1454,11 +1454,11 @@
         <v>1</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12" s="76" t="inlineStr">
         <is>
-          <t>Premiul III</t>
+          <t>Mențiune</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1599,11 +1599,11 @@
         <v>4</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L15" s="76" t="inlineStr">
         <is>
-          <t>Mențiune</t>
+          <t>Membru</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1775,11 +1775,11 @@
         <v>4</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L19" s="76" t="inlineStr">
         <is>
-          <t>Premiul III</t>
+          <t>Mențiune</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1824,11 +1824,11 @@
         <v>1</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L20" s="76" t="inlineStr">
         <is>
-          <t>Premiul III</t>
+          <t>Mențiune</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         <v>7</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L23" s="76" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L25" s="76" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L27" s="76" t="inlineStr">
         <is>
@@ -2182,11 +2182,11 @@
         <v>1</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L28" s="76" t="inlineStr">
         <is>
-          <t>Premiul III</t>
+          <t>Mențiune</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L29" s="76" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L30" s="76" t="inlineStr">
         <is>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L31" s="76" t="inlineStr">
         <is>
@@ -2392,20 +2392,30 @@
           <t>126/100</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n"/>
+      <c r="E33" s="4" t="n">
+        <v>10</v>
+      </c>
       <c r="F33" s="4" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="G33" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H33" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J33" s="4" t="n"/>
-      <c r="K33" s="24" t="n"/>
-      <c r="L33" s="76" t="n"/>
+      <c r="K33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="76" t="inlineStr">
+        <is>
+          <t>Premiul I</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t>6843</t>
@@ -27603,7 +27613,9 @@
           <t>126/100</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
+      <c r="E33" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="6" t="n"/>
       <c r="H33" s="4" t="n"/>
@@ -27783,8 +27795,14 @@
         <f>IF(COUNTA(EE33:FH33)=0, "", COUNTA(EE33:FH33) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE33:FH33))))</f>
         <v/>
       </c>
-      <c r="FK33" s="43" t="n"/>
-      <c r="FL33" s="43" t="n"/>
+      <c r="FK33" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="FL33" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM33" s="43" t="n"/>
       <c r="FN33" s="43" t="n"/>
       <c r="FO33" s="43" t="n"/>
@@ -27803,7 +27821,9 @@
       <c r="GB33" s="4" t="n"/>
       <c r="GC33" s="43" t="n"/>
       <c r="GD33" s="9" t="n"/>
-      <c r="GE33" s="44" t="n"/>
+      <c r="GE33" s="44" t="n">
+        <v>10</v>
+      </c>
       <c r="GF33" s="43" t="n"/>
       <c r="GG33" s="43" t="n"/>
       <c r="GH33" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:41
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2407,7 +2407,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J33" s="4" t="n"/>
+      <c r="J33" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" s="24" t="n">
         <v>1</v>
       </c>
@@ -27617,7 +27619,9 @@
         <v>10</v>
       </c>
       <c r="F33" s="8" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="G33" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="43" t="n"/>
       <c r="J33" s="4" t="n"/>
@@ -27824,7 +27828,11 @@
       <c r="GE33" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="GF33" s="43" t="n"/>
+      <c r="GF33" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="GG33" s="43" t="n"/>
       <c r="GH33" s="43" t="n"/>
       <c r="GI33" s="43" t="n"/>
@@ -49283,8 +49291,12 @@
         </is>
       </c>
       <c r="E33" s="10" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="11" t="n"/>
+      <c r="F33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H33" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:42
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K33" s="24" t="n">
         <v>1</v>
@@ -27620,7 +27620,7 @@
       </c>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="43" t="n"/>
@@ -28194,7 +28194,11 @@
       <c r="SI33" s="4" t="n"/>
       <c r="SJ33" s="4" t="n"/>
       <c r="SK33" s="11" t="n"/>
-      <c r="SL33" s="4" t="n"/>
+      <c r="SL33" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="SM33" s="4" t="n"/>
       <c r="SN33" s="4" t="n"/>
       <c r="SO33" s="4" t="n"/>
@@ -49300,10 +49304,10 @@
       </c>
       <c r="E33" s="10" t="n"/>
       <c r="F33" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H33" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:43
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K33" s="24" t="n">
         <v>1</v>
@@ -45468,7 +45468,9 @@
       </c>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="8" t="n"/>
-      <c r="G33" s="6" t="n"/>
+      <c r="G33" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="43" t="n"/>
       <c r="J33" s="4" t="n"/>
@@ -45608,7 +45610,11 @@
       <c r="EB33" s="9" t="n"/>
       <c r="EC33" s="10" t="n"/>
       <c r="ED33" s="11" t="n"/>
-      <c r="EE33" s="4" t="n"/>
+      <c r="EE33" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="EF33" s="4" t="n"/>
       <c r="EG33" s="4" t="n"/>
       <c r="EH33" s="4" t="n"/>
@@ -49308,10 +49314,10 @@
       </c>
       <c r="E33" s="10" t="n"/>
       <c r="F33" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H33" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:44
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="24" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L30" s="76" t="inlineStr">
         <is>
@@ -2488,20 +2488,30 @@
           <t>128/1</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n"/>
+      <c r="E35" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="F35" s="4" t="n"/>
-      <c r="G35" s="6" t="n"/>
+      <c r="G35" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="H35" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J35" s="4" t="n"/>
-      <c r="K35" s="24" t="n"/>
-      <c r="L35" s="76" t="n"/>
+      <c r="K35" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="L35" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t>9414</t>
@@ -29361,7 +29371,9 @@
           <t>128/1</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n"/>
+      <c r="E35" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="6" t="n"/>
       <c r="H35" s="4" t="n"/>
@@ -29541,8 +29553,14 @@
         <f>IF(COUNTA(EE35:FH35)=0, "", COUNTA(EE35:FH35) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE35:FH35))))</f>
         <v/>
       </c>
-      <c r="FK35" s="43" t="n"/>
-      <c r="FL35" s="43" t="n"/>
+      <c r="FK35" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="FL35" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM35" s="43" t="n"/>
       <c r="FN35" s="43" t="n"/>
       <c r="FO35" s="43" t="n"/>
@@ -29561,7 +29579,9 @@
       <c r="GB35" s="4" t="n"/>
       <c r="GC35" s="43" t="n"/>
       <c r="GD35" s="9" t="n"/>
-      <c r="GE35" s="44" t="n"/>
+      <c r="GE35" s="44" t="n">
+        <v>5</v>
+      </c>
       <c r="GF35" s="43" t="n"/>
       <c r="GG35" s="43" t="n"/>
       <c r="GH35" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:45
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="24" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L30" s="76" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="24" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L35" s="76" t="inlineStr">
         <is>
@@ -2535,20 +2535,30 @@
           <t>128/2</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n"/>
+      <c r="E36" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="F36" s="4" t="n"/>
-      <c r="G36" s="6" t="n"/>
+      <c r="G36" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="H36" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J36" s="4" t="n"/>
-      <c r="K36" s="24" t="n"/>
-      <c r="L36" s="76" t="n"/>
+      <c r="K36" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="L36" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>2250</t>
@@ -30228,11 +30238,19 @@
           <t>128/2</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n"/>
+      <c r="E36" s="6" t="n">
+        <v>6</v>
+      </c>
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="6" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="43" t="n"/>
+      <c r="H36" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I36" s="43" t="inlineStr">
+        <is>
+          <t>25.09</t>
+        </is>
+      </c>
       <c r="J36" s="4" t="n"/>
       <c r="K36" s="43" t="n"/>
       <c r="L36" s="4" t="n"/>
@@ -30251,7 +30269,9 @@
       <c r="Y36" s="43" t="n"/>
       <c r="Z36" s="43" t="n"/>
       <c r="AA36" s="9" t="n"/>
-      <c r="AB36" s="8" t="n"/>
+      <c r="AB36" s="8" t="n">
+        <v>6</v>
+      </c>
       <c r="AC36" s="4" t="n"/>
       <c r="AD36" s="43" t="n"/>
       <c r="AE36" s="4" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:46
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2550,7 +2550,9 @@
           <t>Promovat</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n"/>
+      <c r="J36" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" s="24" t="n">
         <v>11</v>
       </c>
@@ -30242,7 +30244,9 @@
         <v>6</v>
       </c>
       <c r="F36" s="8" t="n"/>
-      <c r="G36" s="6" t="n"/>
+      <c r="G36" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H36" s="4" t="n">
         <v>6</v>
       </c>
@@ -30803,7 +30807,11 @@
       <c r="SI36" s="4" t="n"/>
       <c r="SJ36" s="4" t="n"/>
       <c r="SK36" s="11" t="n"/>
-      <c r="SL36" s="4" t="n"/>
+      <c r="SL36" s="43" t="inlineStr">
+        <is>
+          <t>15.09m</t>
+        </is>
+      </c>
       <c r="SM36" s="4" t="n"/>
       <c r="SN36" s="4" t="n"/>
       <c r="SO36" s="4" t="n"/>
@@ -49461,8 +49469,12 @@
         </is>
       </c>
       <c r="E36" s="10" t="n"/>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="11" t="n"/>
+      <c r="F36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H36" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:47
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2595,7 +2595,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J37" s="4" t="n"/>
+      <c r="J37" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K37" s="24" t="n"/>
       <c r="L37" s="76" t="n"/>
       <c r="M37" t="inlineStr">
@@ -31105,7 +31107,9 @@
       </c>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="8" t="n"/>
-      <c r="G37" s="6" t="n"/>
+      <c r="G37" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="43" t="n"/>
       <c r="J37" s="4" t="n"/>
@@ -31304,7 +31308,11 @@
       <c r="GC37" s="43" t="n"/>
       <c r="GD37" s="9" t="n"/>
       <c r="GE37" s="44" t="n"/>
-      <c r="GF37" s="43" t="n"/>
+      <c r="GF37" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="GG37" s="43" t="n"/>
       <c r="GH37" s="43" t="n"/>
       <c r="GI37" s="43" t="n"/>
@@ -49501,8 +49509,12 @@
         </is>
       </c>
       <c r="E37" s="10" t="n"/>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="F37" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H37" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:48
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K37" s="24" t="n"/>
       <c r="L37" s="76" t="n"/>
@@ -31108,7 +31108,7 @@
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="43" t="n"/>
@@ -31788,7 +31788,11 @@
       <c r="WK37" s="4" t="n"/>
       <c r="WL37" s="4" t="n"/>
       <c r="WM37" s="11" t="n"/>
-      <c r="WN37" s="4" t="n"/>
+      <c r="WN37" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="WO37" s="4" t="n"/>
       <c r="WP37" s="4" t="n"/>
       <c r="WQ37" s="4" t="n"/>
@@ -49514,10 +49518,10 @@
       </c>
       <c r="E37" s="10" t="n"/>
       <c r="F37" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:49
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2634,7 +2634,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J38" s="4" t="n"/>
+      <c r="J38" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K38" s="24" t="n"/>
       <c r="L38" s="76" t="n"/>
       <c r="M38" t="inlineStr">
@@ -31968,7 +31970,9 @@
       </c>
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="8" t="n"/>
-      <c r="G38" s="6" t="n"/>
+      <c r="G38" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="43" t="n"/>
       <c r="J38" s="4" t="n"/>
@@ -32285,7 +32289,11 @@
       <c r="KE38" s="9" t="n"/>
       <c r="KF38" s="43" t="n"/>
       <c r="KG38" s="44" t="n"/>
-      <c r="KH38" s="43" t="n"/>
+      <c r="KH38" s="43" t="inlineStr">
+        <is>
+          <t>24.09m</t>
+        </is>
+      </c>
       <c r="KI38" s="43" t="n"/>
       <c r="KJ38" s="43" t="n"/>
       <c r="KK38" s="43" t="n"/>
@@ -49549,8 +49557,12 @@
         </is>
       </c>
       <c r="E38" s="10" t="n"/>
-      <c r="F38" s="9" t="n"/>
-      <c r="G38" s="11" t="n"/>
+      <c r="F38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H38" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:50
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K38" s="24" t="n"/>
       <c r="L38" s="76" t="n"/>
@@ -47449,7 +47449,9 @@
       </c>
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="8" t="n"/>
-      <c r="G38" s="6" t="n"/>
+      <c r="G38" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="43" t="n"/>
       <c r="J38" s="4" t="n"/>
@@ -47648,7 +47650,11 @@
       <c r="GC38" s="4" t="n"/>
       <c r="GD38" s="4" t="n"/>
       <c r="GE38" s="11" t="n"/>
-      <c r="GF38" s="4" t="n"/>
+      <c r="GF38" s="43" t="inlineStr">
+        <is>
+          <t>21.09m</t>
+        </is>
+      </c>
       <c r="GG38" s="4" t="n"/>
       <c r="GH38" s="4" t="n"/>
       <c r="GI38" s="4" t="n"/>
@@ -49566,10 +49572,10 @@
       </c>
       <c r="E38" s="10" t="n"/>
       <c r="F38" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H38" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:51
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2710,7 +2710,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J40" s="4" t="n"/>
+      <c r="J40" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
       <c r="M40" t="inlineStr">
@@ -33678,7 +33680,9 @@
       </c>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
-      <c r="G40" s="6" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
       <c r="J40" s="4" t="n"/>
@@ -33700,7 +33704,11 @@
       <c r="Z40" s="43" t="n"/>
       <c r="AA40" s="9" t="n"/>
       <c r="AB40" s="8" t="n"/>
-      <c r="AC40" s="4" t="n"/>
+      <c r="AC40" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="AD40" s="43" t="n"/>
       <c r="AE40" s="4" t="n"/>
       <c r="AF40" s="43" t="n"/>
@@ -49639,8 +49647,12 @@
         </is>
       </c>
       <c r="E40" s="10" t="n"/>
-      <c r="F40" s="9" t="n"/>
-      <c r="G40" s="11" t="n"/>
+      <c r="F40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="H40" s="11" t="n">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:52
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -33681,7 +33681,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -33709,7 +33709,11 @@
           <t>25.09m</t>
         </is>
       </c>
-      <c r="AD40" s="43" t="n"/>
+      <c r="AD40" s="43" t="inlineStr">
+        <is>
+          <t>28.09m</t>
+        </is>
+      </c>
       <c r="AE40" s="4" t="n"/>
       <c r="AF40" s="43" t="n"/>
       <c r="AG40" s="4" t="n"/>
@@ -49648,10 +49652,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:53
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -33681,7 +33681,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -33952,7 +33952,11 @@
       <c r="ID40" s="10" t="n"/>
       <c r="IE40" s="4" t="n"/>
       <c r="IF40" s="44" t="n"/>
-      <c r="IG40" s="4" t="n"/>
+      <c r="IG40" s="43" t="inlineStr">
+        <is>
+          <t>21.09m</t>
+        </is>
+      </c>
       <c r="IH40" s="43" t="n"/>
       <c r="II40" s="4" t="n"/>
       <c r="IJ40" s="43" t="n"/>
@@ -49656,10 +49660,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:54
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -33681,7 +33681,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -34259,7 +34259,11 @@
       <c r="SI40" s="4" t="n"/>
       <c r="SJ40" s="4" t="n"/>
       <c r="SK40" s="11" t="n"/>
-      <c r="SL40" s="4" t="n"/>
+      <c r="SL40" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="SM40" s="4" t="n"/>
       <c r="SN40" s="4" t="n"/>
       <c r="SO40" s="4" t="n"/>
@@ -49668,10 +49672,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:55
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -33681,7 +33681,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -34381,7 +34381,11 @@
       <c r="WK40" s="4" t="n"/>
       <c r="WL40" s="4" t="n"/>
       <c r="WM40" s="11" t="n"/>
-      <c r="WN40" s="4" t="n"/>
+      <c r="WN40" s="43" t="inlineStr">
+        <is>
+          <t>25.09m</t>
+        </is>
+      </c>
       <c r="WO40" s="4" t="n"/>
       <c r="WP40" s="4" t="n"/>
       <c r="WQ40" s="4" t="n"/>
@@ -49676,10 +49680,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:56
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -48254,7 +48254,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -48459,7 +48459,11 @@
           <t>23.09m</t>
         </is>
       </c>
-      <c r="GG40" s="4" t="n"/>
+      <c r="GG40" s="43" t="inlineStr">
+        <is>
+          <t>24.09m</t>
+        </is>
+      </c>
       <c r="GH40" s="4" t="n"/>
       <c r="GI40" s="4" t="n"/>
       <c r="GJ40" s="4" t="n"/>
@@ -49686,10 +49690,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 12:57
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K40" s="24" t="n"/>
       <c r="L40" s="76" t="n"/>
@@ -48254,7 +48254,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="43" t="n"/>
@@ -48395,7 +48395,11 @@
       <c r="EB40" s="9" t="n"/>
       <c r="EC40" s="10" t="n"/>
       <c r="ED40" s="11" t="n"/>
-      <c r="EE40" s="4" t="n"/>
+      <c r="EE40" s="43" t="inlineStr">
+        <is>
+          <t>22.09m</t>
+        </is>
+      </c>
       <c r="EF40" s="4" t="n"/>
       <c r="EG40" s="4" t="n"/>
       <c r="EH40" s="4" t="n"/>
@@ -49694,10 +49698,10 @@
       </c>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H40" s="11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Update automat catalog: 28.09.2026 17:08
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -37239,10 +37239,10 @@
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="6" t="n"/>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="43" t="n"/>
       <c r="J11" s="4" t="n"/>
@@ -37443,7 +37443,7 @@
       <c r="GE11" s="11" t="n"/>
       <c r="GF11" s="43" t="inlineStr">
         <is>
-          <t>21.09</t>
+          <t>21.09m</t>
         </is>
       </c>
       <c r="GG11" s="4" t="n"/>
@@ -48798,10 +48798,10 @@
           <t>126/78</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="9" t="n"/>
       <c r="G11" s="11" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Update automat catalog: 02.10.2026 10:00
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -2259,30 +2259,20 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
-        <v>4</v>
-      </c>
+      <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
-      <c r="G30" s="6" t="n">
-        <v>4</v>
-      </c>
+      <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Corigent / Repetent</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="L30" s="76" t="inlineStr">
-        <is>
-          <t>Membru</t>
-        </is>
-      </c>
+      <c r="K30" s="24" t="n"/>
+      <c r="L30" s="76" t="n"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>7508</t>
@@ -25086,9 +25076,7 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n">
-        <v>4</v>
-      </c>
+      <c r="E30" s="6" t="n"/>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n"/>
@@ -25268,14 +25256,8 @@
         <f>IF(COUNTA(EE30:FH30)=0, "", COUNTA(EE30:FH30) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE30:FH30))))</f>
         <v/>
       </c>
-      <c r="FK30" s="43" t="n">
-        <v>4</v>
-      </c>
-      <c r="FL30" s="43" t="inlineStr">
-        <is>
-          <t>18.09</t>
-        </is>
-      </c>
+      <c r="FK30" s="43" t="n"/>
+      <c r="FL30" s="43" t="n"/>
       <c r="FM30" s="43" t="n"/>
       <c r="FN30" s="43" t="n"/>
       <c r="FO30" s="43" t="n"/>
@@ -25294,9 +25276,7 @@
       <c r="GB30" s="4" t="n"/>
       <c r="GC30" s="43" t="n"/>
       <c r="GD30" s="9" t="n"/>
-      <c r="GE30" s="44" t="n">
-        <v>4</v>
-      </c>
+      <c r="GE30" s="44" t="n"/>
       <c r="GF30" s="43" t="n"/>
       <c r="GG30" s="43" t="n"/>
       <c r="GH30" s="43" t="n"/>

</xml_diff>

<commit_message>
Update automat catalog: 02.10.2026 10:02
</commit_message>
<xml_diff>
--- a/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
+++ b/catalog_scolar_clasa_IX_TH_Turda-v15.xlsx
@@ -1503,7 +1503,7 @@
         <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" s="76" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L17" s="76" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         <v>6</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L21" s="76" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         <v>7</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L23" s="76" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L25" s="76" t="inlineStr">
         <is>
@@ -2133,7 +2133,7 @@
       </c>
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L27" s="76" t="inlineStr">
         <is>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L29" s="76" t="inlineStr">
         <is>
@@ -2259,20 +2259,30 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n"/>
+      <c r="E30" s="4" t="n">
+        <v>8</v>
+      </c>
       <c r="F30" s="4" t="n"/>
-      <c r="G30" s="6" t="n"/>
+      <c r="G30" s="6" t="n">
+        <v>8</v>
+      </c>
       <c r="H30" s="4" t="n">
         <v>10</v>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promovat</t>
         </is>
       </c>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="24" t="n"/>
-      <c r="L30" s="76" t="n"/>
+      <c r="K30" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="L30" s="76" t="inlineStr">
+        <is>
+          <t>Membru</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>7508</t>
@@ -2313,7 +2323,7 @@
       </c>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L31" s="76" t="inlineStr">
         <is>
@@ -2448,7 +2458,7 @@
       </c>
       <c r="J34" s="4" t="n"/>
       <c r="K34" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L34" s="76" t="inlineStr">
         <is>
@@ -2495,7 +2505,7 @@
       </c>
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L35" s="76" t="inlineStr">
         <is>
@@ -2544,7 +2554,7 @@
         <v>1</v>
       </c>
       <c r="K36" s="24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L36" s="76" t="inlineStr">
         <is>
@@ -25076,7 +25086,9 @@
           <t>126/97</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
+      <c r="E30" s="6" t="n">
+        <v>8</v>
+      </c>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="4" t="n"/>
@@ -25256,8 +25268,14 @@
         <f>IF(COUNTA(EE30:FH30)=0, "", COUNTA(EE30:FH30) - SUMPRODUCT(--ISNUMBER(SEARCH("m", EE30:FH30))))</f>
         <v/>
       </c>
-      <c r="FK30" s="43" t="n"/>
-      <c r="FL30" s="43" t="n"/>
+      <c r="FK30" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="FL30" s="43" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
       <c r="FM30" s="43" t="n"/>
       <c r="FN30" s="43" t="n"/>
       <c r="FO30" s="43" t="n"/>
@@ -25276,7 +25294,9 @@
       <c r="GB30" s="4" t="n"/>
       <c r="GC30" s="43" t="n"/>
       <c r="GD30" s="9" t="n"/>
-      <c r="GE30" s="44" t="n"/>
+      <c r="GE30" s="44" t="n">
+        <v>8</v>
+      </c>
       <c r="GF30" s="43" t="n"/>
       <c r="GG30" s="43" t="n"/>
       <c r="GH30" s="43" t="n"/>

</xml_diff>